<commit_message>
actualización productos Chaquetas equipos
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0526577688ca4eec/Escritorio/Proyectos developer/Diseños_Gasper/Back-end/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="580" documentId="8_{ADBBDD1F-37F2-455A-919D-03174E12E1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05BC9152-A612-4427-9C22-BE0904F86F93}"/>
+  <xr:revisionPtr revIDLastSave="603" documentId="8_{ADBBDD1F-37F2-455A-919D-03174E12E1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96655D59-78B5-465D-9B25-EE346B63AC3C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -332,12 +332,6 @@
   </si>
   <si>
     <t>{"yellow":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270323/p6k7eqjzznst2bxrg2vz.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270317/t5cdbjnctbumlg675bnh.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270319/lggiyj7ykumexocgdg3w.png"],"blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270300/dph8v8zxcw4oobwmchp6.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270300/wheagvkqjkcca47yvhlb.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270301/fo3oopc2w4gguhsxbwky.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270308/gtl37zjvfml3vmuv2o9l.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270313/z5kuunpfvxclcend8okq.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270310/kk0wsleipwg1z2mbcqku.png"],"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270304/hl9fado9nquhxaicselq.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270305/ru5vmxdsif5kt61snx2u.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270306/vodvrpkiopfd6onb91ix.png"],"green":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270311/ku0bx9n4tm9yljlo0wf7.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270321/ojw3mz6n6hix4ube3qne.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270316/fg6dnjtwpxwm4hoghz91.png"],"orange":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270325/eduy6ep0xxc17tqusqq2.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270329/gvwagkni5jgyouq7z2oc.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270326/r9qvdtgbdeyir30bac22.png"],"royalblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270330/z2mavjespmfokq9blbck.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270335/amahc57ashuhn1en1uus.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270333/uqc0lg7dkqsbpk9lul2p.png"],"mediumblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270341/fmj9dftl1oejpyyv9f5e.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270341/nc1781x31vupdepm9piz.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773270343/kh5eadc7awmjbgrychhh.png"]}</t>
-  </si>
-  <si>
-    <t>black,white,blue,royalblue,mediumblue,green,darkgreen,palegreen,red,crimson</t>
-  </si>
-  <si>
-    <t>{"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251884/ec6qea5mjwajn6nk0dln.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251877/hkcop8xbp6padhtnueg5.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251881/u3sf21qmczzhmkc9chvn.png"],"white":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252051/kklwfmuzcbmquhjwr1le.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252055/gj58jpkwmgolvaueqotb.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252059/txlffqcfnjip066ftd8k.png"],"blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251911/jsswfj3yfpgbp0fneaot.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251916/jnbw9puupo8igk8ff0lv.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251920/zkn50gnfqb1ab9knzrtr.png"],"royalblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252003/arjirrtfe28hrruk98by.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252007/aeprferwkxtmejtmbnt4.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252011/o5ppb5ekeva72tecdsb6.png"],"mediumblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251888/cnlog1ryadij1b1nfw4o.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251892/rbhc0i968a6azm11l6kd.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251896/dmpmycsic51qpiehjzze.png"],"green":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252026/lu0evxujmcpajk0alk78.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252030/p1jsjnd3p5sah6f8yzfd.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252039/m9pzvfpixsmhbu9hmv6n.png"],"darkgreen":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252062/fmoab07kdfbqnzoh0cfe.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252066/gcx3hzyojzuimxllhakv.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252071/jotsfswaol54s09fbfsm.png"],"palegreen":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252034/nnvtss7oi7g69wu0jljp.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252042/cm0q4cexpjve8e1m8quj.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252047/gogphkry0pzgvwsbz7q5.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252015/p1arccwljiinxatuwq2z.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252018/iafldqth4txewfsqgm3h.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252022/ndnjgaf5il8pc2oos882.png"],"crimson":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251899/tvxqa3edphyb1hdrtmsh.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251903/o9hsbfufrpx0n2n2budn.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251907/hgknyxcfxcewldkkz0a2.png"]}</t>
   </si>
   <si>
     <t>olive,red,green,blue,crimson,purple,yellow</t>
@@ -1640,6 +1634,58 @@
     "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421890/s6aqfmvqvxzxbrea9o6m.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421845/vbi5lsovyoekcxcmdedi.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421982/wsanluxtsjfru3qedb6i.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421995/l7d62rcgfwbdhch3exdo.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421897/eetddm28orkox7hoyivc.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421842/sswalmqkan70tvt5xbb5.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421987/axmuavtqpl5qzkfbifns.png" ],
   "hotpink": [
     "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773422004/ybytqypmgep2zvvafglf.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421915/b4pr9artbraayulde8qo.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421836/zqp4tqcz5p3yqok4yz1a.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421839/nbewqlcmyzgwkgckqqqg.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421822/cyjggxc3enonwvqb70se.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421854/gcim37vumhuin6espkxf.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421947/op6q7fj0zfvej8zz7jfm.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773422006/njr7jg5mujkmadzle1gz.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421951/rzxqpkwtzyttbwocwuaj.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421966/aypwbrl04yespk7dat5r.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421962/l4mtufoby7nwglrfueng.png"   ]}</t>
+  </si>
+  <si>
+    <t>{
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874935/obukza5vd0lbczqa3jmj.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874935/xieyxnibupu7gyqbottu.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251916/jnbw9puupo8igk8ff0lv.png"
+  ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874935/vut0fklpq9iq9pgvq0qu.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251903/o9hsbfufrpx0n2n2budn.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874936/nnnnksosglnwfxheeugo.png"
+  ],
+  "white": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874937/ekjfmubhng4unim5sk2n.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252055/gj58jpkwmgolvaueqotb.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252059/txlffqcfnjip066ftd8k.png"
+  ],
+  "darkgreen": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252026/lu0evxujmcpajk0alk78.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252030/p1jsjnd3p5sah6f8yzfd.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252039/m9pzvfpixsmhbu9hmv6n.png"
+  ],
+  "black": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874935/xhdaskfvjrjb2gdztdvl.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251892/rbhc0i968a6azm11l6kd.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874935/p1qxnyky6zo2pxzhwxil.png"
+  ],
+  "darkred": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874936/vepamtjmc71hnjdflqq0.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773251881/u3sf21qmczzhmkc9chvn.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874934/mxp2otdhyeefdiccxrml.png"
+  ],
+  "palegreen": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874938/oyyrvqngbzkjcd4nx1gp.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252042/cm0q4cexpjve8e1m8quj.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252047/gogphkry0pzgvwsbz7q5.png"
+  ],
+  "crimson": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252062/fmoab07kdfbqnzoh0cfe.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252066/gcx3hzyojzuimxllhakv.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252071/jotsfswaol54s09fbfsm.png"
+  ],
+   "mediumblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252003/arjirrtfe28hrruk98by.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252007/aeprferwkxtmejtmbnt4.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773252011/o5ppb5ekeva72tecdsb6.png"
+  ],  "olive": ["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874936/gepqc6gvitwzvgsxy2ok.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773874937/qavzumaav2irbqpfkhha.png" ]
+}</t>
+  </si>
+  <si>
+    <t>blue,red,white,darkgreen,black,darkred,palegreen,crimson,mediumblue,olive</t>
   </si>
 </sst>
 </file>
@@ -2137,7 +2183,7 @@
         <v>16</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>11</v>
@@ -2169,10 +2215,10 @@
     </row>
     <row r="3" spans="1:11" s="3" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>18</v>
+        <v>177</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>11</v>
@@ -2200,31 +2246,33 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="3" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" s="3" customFormat="1" ht="89.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="6">
-        <v>21000</v>
-      </c>
-      <c r="E4" s="6"/>
+        <v>28000</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>35</v>
+      </c>
       <c r="F4" s="6">
-        <v>31500</v>
+        <v>42000</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>72</v>
+        <v>17</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>74</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J4" s="6" t="b">
         <v>0</v>
@@ -2233,15 +2281,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11" s="3" customFormat="1" ht="89.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" s="3" customFormat="1" ht="145" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>178</v>
+        <v>19</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D5" s="6">
         <v>28000</v>
@@ -2256,10 +2304,10 @@
         <v>17</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J5" s="6" t="b">
         <v>0</v>
@@ -2268,33 +2316,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" s="3" customFormat="1" ht="145" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="118.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D6" s="6">
-        <v>28000</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>35</v>
-      </c>
+        <v>21000</v>
+      </c>
+      <c r="E6" s="6"/>
       <c r="F6" s="6">
-        <v>42000</v>
+        <v>33000</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>77</v>
+        <v>139</v>
       </c>
       <c r="J6" s="6" t="b">
         <v>0</v>
@@ -2303,31 +2349,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="118.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="77.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="6">
-        <v>21000</v>
-      </c>
-      <c r="E7" s="6"/>
+        <v>33000</v>
+      </c>
+      <c r="E7" s="7"/>
       <c r="F7" s="6">
-        <v>33000</v>
+        <v>49500</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>141</v>
+        <v>78</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>80</v>
       </c>
       <c r="J7" s="6" t="b">
         <v>0</v>
@@ -2336,31 +2382,33 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="77.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="6">
-        <v>33000</v>
-      </c>
-      <c r="E8" s="7"/>
+        <v>20000</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>36</v>
+      </c>
       <c r="F8" s="6">
-        <v>49500</v>
+        <v>30000</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="J8" s="6" t="b">
         <v>0</v>
@@ -2371,10 +2419,10 @@
     </row>
     <row r="9" spans="1:11" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>23</v>
+        <v>178</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>163</v>
+        <v>183</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>11</v>
@@ -2404,33 +2452,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>180</v>
+        <v>24</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D10" s="6">
-        <v>20000</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>36</v>
-      </c>
+        <v>18000</v>
+      </c>
+      <c r="E10" s="6"/>
       <c r="F10" s="6">
-        <v>30000</v>
+        <v>27000</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="I10" s="11" t="s">
-        <v>82</v>
+        <v>14</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>84</v>
       </c>
       <c r="J10" s="6" t="b">
         <v>0</v>
@@ -2441,10 +2487,10 @@
     </row>
     <row r="11" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>24</v>
+        <v>179</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>163</v>
+        <v>183</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>11</v>
@@ -2472,31 +2518,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="47" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>181</v>
+        <v>85</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="6">
-        <v>18000</v>
+        <v>21000</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6">
-        <v>27000</v>
+        <v>31000</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="I12" s="12" t="s">
-        <v>84</v>
+        <v>86</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>140</v>
       </c>
       <c r="J12" s="6" t="b">
         <v>0</v>
@@ -2507,10 +2553,10 @@
     </row>
     <row r="13" spans="1:11" ht="47" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>85</v>
+        <v>180</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>11</v>
@@ -2529,7 +2575,7 @@
         <v>86</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="J13" s="6" t="b">
         <v>0</v>
@@ -2538,31 +2584,33 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="47" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="D14" s="6">
-        <v>21000</v>
-      </c>
-      <c r="E14" s="6"/>
+        <v>38000</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>37</v>
+      </c>
       <c r="F14" s="6">
-        <v>31000</v>
+        <v>57000</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="I14" s="11" t="s">
-        <v>142</v>
+        <v>87</v>
+      </c>
+      <c r="I14" s="12" t="s">
+        <v>141</v>
       </c>
       <c r="J14" s="6" t="b">
         <v>0</v>
@@ -2573,10 +2621,10 @@
     </row>
     <row r="15" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>163</v>
+        <v>183</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>27</v>
@@ -2597,7 +2645,7 @@
         <v>87</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J15" s="6" t="b">
         <v>0</v>
@@ -2608,13 +2656,13 @@
     </row>
     <row r="16" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="D16" s="6">
         <v>38000</v>
@@ -2632,7 +2680,7 @@
         <v>87</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J16" s="6" t="b">
         <v>0</v>
@@ -2643,10 +2691,10 @@
     </row>
     <row r="17" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>163</v>
+        <v>183</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>11</v>
@@ -2667,7 +2715,7 @@
         <v>87</v>
       </c>
       <c r="I17" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J17" s="6" t="b">
         <v>0</v>
@@ -2676,33 +2724,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
-        <v>167</v>
+        <v>25</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D18" s="6">
-        <v>38000</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>37</v>
-      </c>
+        <v>21000</v>
+      </c>
+      <c r="E18" s="6"/>
       <c r="F18" s="6">
-        <v>57000</v>
+        <v>31500</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I18" s="12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J18" s="6" t="b">
         <v>0</v>
@@ -2713,10 +2759,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>25</v>
+        <v>162</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>163</v>
+        <v>10</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>30</v>
@@ -2735,7 +2781,7 @@
         <v>88</v>
       </c>
       <c r="I19" s="12" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J19" s="6" t="b">
         <v>0</v>
@@ -2744,31 +2790,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>10</v>
+        <v>161</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D20" s="6">
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="6">
-        <v>31500</v>
+        <v>28000</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>88</v>
+        <v>14</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>89</v>
       </c>
       <c r="I20" s="12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J20" s="6" t="b">
         <v>0</v>
@@ -2779,10 +2825,10 @@
     </row>
     <row r="21" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
-        <v>168</v>
+        <v>29</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>163</v>
+        <v>183</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>11</v>
@@ -2801,7 +2847,7 @@
         <v>89</v>
       </c>
       <c r="I21" s="12" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J21" s="6" t="b">
         <v>0</v>
@@ -2810,28 +2856,28 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" ht="54.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D22" s="6">
-        <v>22000</v>
+        <v>21000</v>
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="6">
-        <v>28000</v>
+        <v>31500</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>89</v>
+        <v>145</v>
       </c>
       <c r="I22" s="12" t="s">
         <v>146</v>
@@ -2843,31 +2889,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="54.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D23" s="6">
-        <v>21000</v>
+        <v>47000</v>
       </c>
       <c r="E23" s="6"/>
       <c r="F23" s="6">
-        <v>31500</v>
+        <v>70500</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H23" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="I23" s="12" t="s">
         <v>147</v>
-      </c>
-      <c r="I23" s="12" t="s">
-        <v>148</v>
       </c>
       <c r="J23" s="6" t="b">
         <v>0</v>
@@ -2878,29 +2924,29 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D24" s="6">
-        <v>47000</v>
+        <v>25000</v>
       </c>
       <c r="E24" s="6"/>
       <c r="F24" s="6">
-        <v>70500</v>
+        <v>37500</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I24" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J24" s="6" t="b">
         <v>0</v>
@@ -2911,29 +2957,29 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D25" s="6">
-        <v>25000</v>
+        <v>22000</v>
       </c>
       <c r="E25" s="6"/>
       <c r="F25" s="6">
-        <v>37500</v>
+        <v>33000</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>150</v>
+        <v>93</v>
       </c>
       <c r="J25" s="6" t="b">
         <v>0</v>
@@ -2944,10 +2990,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
-        <v>39</v>
+        <v>167</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>185</v>
+        <v>10</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>11</v>
@@ -2975,31 +3021,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
-        <v>169</v>
+        <v>18</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>10</v>
+        <v>183</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D27" s="6">
-        <v>22000</v>
+        <v>21000</v>
       </c>
       <c r="E27" s="6"/>
       <c r="F27" s="6">
-        <v>33000</v>
+        <v>31500</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H27" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="I27" s="12" t="s">
-        <v>93</v>
+      <c r="H27" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="J27" s="6" t="b">
         <v>0</v>
@@ -3013,7 +3059,7 @@
         <v>40</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>11</v>
@@ -3043,7 +3089,7 @@
     </row>
     <row r="29" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>10</v>
@@ -3065,7 +3111,7 @@
         <v>96</v>
       </c>
       <c r="I29" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J29" s="6" t="b">
         <v>0</v>
@@ -3076,7 +3122,7 @@
     </row>
     <row r="30" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>10</v>
@@ -3177,7 +3223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" ht="55.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
         <v>47</v>
       </c>
@@ -3198,10 +3244,10 @@
         <v>14</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="I33" s="12" t="s">
-        <v>104</v>
+        <v>237</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>236</v>
       </c>
       <c r="J33" s="6" t="b">
         <v>0</v>
@@ -3231,10 +3277,10 @@
         <v>14</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I34" s="12" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="J34" s="6" t="b">
         <v>0</v>
@@ -3245,7 +3291,7 @@
     </row>
     <row r="35" spans="1:11" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>10</v>
@@ -3257,7 +3303,7 @@
         <v>17000</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F35" s="6">
         <v>34000</v>
@@ -3266,10 +3312,10 @@
         <v>41</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J35" s="6" t="b">
         <v>0</v>
@@ -3280,7 +3326,7 @@
     </row>
     <row r="36" spans="1:11" ht="126.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>10</v>
@@ -3292,7 +3338,7 @@
         <v>17000</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F36" s="6">
         <v>34000</v>
@@ -3301,10 +3347,10 @@
         <v>41</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="J36" s="6" t="b">
         <v>0</v>
@@ -3315,7 +3361,7 @@
     </row>
     <row r="37" spans="1:11" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>10</v>
@@ -3327,7 +3373,7 @@
         <v>17000</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F37" s="6">
         <v>34000</v>
@@ -3336,10 +3382,10 @@
         <v>41</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="J37" s="6" t="b">
         <v>0</v>
@@ -3350,7 +3396,7 @@
     </row>
     <row r="38" spans="1:11" ht="91" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="6" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>10</v>
@@ -3362,7 +3408,7 @@
         <v>17000</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F38" s="6">
         <v>34000</v>
@@ -3371,10 +3417,10 @@
         <v>41</v>
       </c>
       <c r="H38" s="7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I38" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J38" s="6" t="b">
         <v>0</v>
@@ -3385,7 +3431,7 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>10</v>
@@ -3404,10 +3450,10 @@
         <v>52</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J39" s="6" t="b">
         <v>0</v>
@@ -3437,10 +3483,10 @@
         <v>52</v>
       </c>
       <c r="H40" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="I40" s="13" t="s">
         <v>114</v>
-      </c>
-      <c r="I40" s="13" t="s">
-        <v>116</v>
       </c>
       <c r="J40" s="6" t="b">
         <v>0</v>
@@ -3470,10 +3516,10 @@
         <v>14</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="I41" s="14" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="J41" s="6" t="b">
         <v>0</v>
@@ -3484,7 +3530,7 @@
     </row>
     <row r="42" spans="1:11" ht="98.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>10</v>
@@ -3503,10 +3549,10 @@
         <v>45</v>
       </c>
       <c r="H42" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I42" s="15" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J42" s="6" t="b">
         <v>0</v>
@@ -3536,10 +3582,10 @@
         <v>45</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I43" s="15" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J43" s="6" t="b">
         <v>0</v>
@@ -3569,10 +3615,10 @@
         <v>14</v>
       </c>
       <c r="H44" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I44" s="8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="J44" s="6" t="b">
         <v>0</v>
@@ -3604,10 +3650,10 @@
         <v>56</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="J45" s="6" t="b">
         <v>0</v>
@@ -3637,10 +3683,10 @@
         <v>59</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I46" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J46" s="6" t="b">
         <v>0</v>
@@ -3670,10 +3716,10 @@
         <v>13</v>
       </c>
       <c r="H47" s="15" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I47" s="15" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J47" s="6" t="b">
         <v>0</v>
@@ -3684,7 +3730,7 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="6" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>10</v>
@@ -3703,10 +3749,10 @@
         <v>61</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I48" s="14" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="J48" s="6" t="b">
         <v>0</v>
@@ -3736,10 +3782,10 @@
         <v>12</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="J49" s="6" t="b">
         <v>0</v>
@@ -3753,7 +3799,7 @@
         <v>63</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>11</v>
@@ -3769,10 +3815,10 @@
         <v>12</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I50" s="14" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J50" s="6" t="b">
         <v>0</v>
@@ -3802,10 +3848,10 @@
         <v>12</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I51" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J51" s="6" t="b">
         <v>0</v>
@@ -3835,10 +3881,10 @@
         <v>14</v>
       </c>
       <c r="H52" s="15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I52" s="15" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="J52" s="6" t="b">
         <v>0</v>
@@ -3852,7 +3898,7 @@
         <v>66</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>11</v>
@@ -3868,10 +3914,10 @@
         <v>14</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I53" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J53" s="6" t="b">
         <v>0</v>
@@ -3885,7 +3931,7 @@
         <v>67</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>11</v>
@@ -3901,10 +3947,10 @@
         <v>14</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J54" s="6" t="b">
         <v>0</v>
@@ -3918,7 +3964,7 @@
         <v>68</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>11</v>
@@ -3934,10 +3980,10 @@
         <v>14</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="J55" s="6" t="b">
         <v>0</v>
@@ -3951,7 +3997,7 @@
         <v>69</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>11</v>
@@ -3967,10 +4013,10 @@
         <v>32</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="J56" s="6" t="b">
         <v>0</v>
@@ -3981,10 +4027,10 @@
     </row>
     <row r="57" spans="1:11" ht="377" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>11</v>
@@ -3993,7 +4039,7 @@
         <v>22000</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F57" s="6">
         <v>27000</v>
@@ -4002,10 +4048,10 @@
         <v>17</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="I57" s="15" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="J57" s="6" t="b">
         <v>0</v>
@@ -4016,10 +4062,10 @@
     </row>
     <row r="58" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A58" s="16" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B58" s="16" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C58" s="16" t="s">
         <v>27</v>
@@ -4035,10 +4081,10 @@
         <v>14</v>
       </c>
       <c r="H58" s="17" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="I58" s="18" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="J58" s="19" t="b">
         <v>0</v>
@@ -4049,10 +4095,10 @@
     </row>
     <row r="59" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A59" s="16" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C59" s="16" t="s">
         <v>20</v>
@@ -4068,10 +4114,10 @@
         <v>14</v>
       </c>
       <c r="H59" s="17" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="I59" s="18" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="J59" s="19" t="b">
         <v>0</v>
@@ -4082,10 +4128,10 @@
     </row>
     <row r="60" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A60" s="16" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B60" s="16" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C60" s="16" t="s">
         <v>20</v>
@@ -4101,10 +4147,10 @@
         <v>14</v>
       </c>
       <c r="H60" s="17" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="I60" s="18" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="J60" s="19" t="b">
         <v>0</v>
@@ -4115,10 +4161,10 @@
     </row>
     <row r="61" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A61" s="16" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B61" s="16" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C61" s="16" t="s">
         <v>20</v>
@@ -4134,10 +4180,10 @@
         <v>14</v>
       </c>
       <c r="H61" s="17" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="I61" s="18" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J61" s="19" t="b">
         <v>0</v>
@@ -4148,10 +4194,10 @@
     </row>
     <row r="62" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A62" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B62" s="16" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C62" s="16" t="s">
         <v>20</v>
@@ -4167,10 +4213,10 @@
         <v>14</v>
       </c>
       <c r="H62" s="17" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="I62" s="18" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J62" s="19" t="b">
         <v>0</v>
@@ -4181,10 +4227,10 @@
     </row>
     <row r="63" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A63" s="16" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B63" s="16" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C63" s="16" t="s">
         <v>20</v>
@@ -4200,10 +4246,10 @@
         <v>14</v>
       </c>
       <c r="H63" s="17" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="I63" s="18" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="J63" s="19" t="b">
         <v>0</v>
@@ -4214,10 +4260,10 @@
     </row>
     <row r="64" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A64" s="16" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B64" s="16" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C64" s="16" t="s">
         <v>20</v>
@@ -4233,10 +4279,10 @@
         <v>14</v>
       </c>
       <c r="H64" s="17" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I64" s="18" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="J64" s="19" t="b">
         <v>0</v>
@@ -4247,10 +4293,10 @@
     </row>
     <row r="65" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A65" s="16" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B65" s="16" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C65" s="16" t="s">
         <v>20</v>
@@ -4266,10 +4312,10 @@
         <v>14</v>
       </c>
       <c r="H65" s="17" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I65" s="18" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="J65" s="19" t="b">
         <v>0</v>
@@ -4280,10 +4326,10 @@
     </row>
     <row r="66" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A66" s="16" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B66" s="16" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C66" s="16" t="s">
         <v>20</v>
@@ -4299,10 +4345,10 @@
         <v>14</v>
       </c>
       <c r="H66" s="17" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="I66" s="18" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="J66" s="19" t="b">
         <v>0</v>
@@ -4313,10 +4359,10 @@
     </row>
     <row r="67" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A67" s="16" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B67" s="16" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C67" s="16" t="s">
         <v>20</v>
@@ -4332,10 +4378,10 @@
         <v>14</v>
       </c>
       <c r="H67" s="17" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="I67" s="18" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="J67" s="19" t="b">
         <v>0</v>
@@ -4346,10 +4392,10 @@
     </row>
     <row r="68" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A68" s="16" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B68" s="16" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C68" s="16" t="s">
         <v>20</v>
@@ -4365,10 +4411,10 @@
         <v>14</v>
       </c>
       <c r="H68" s="17" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="I68" s="18" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="J68" s="19" t="b">
         <v>0</v>
@@ -4379,10 +4425,10 @@
     </row>
     <row r="69" spans="1:11" ht="406" x14ac:dyDescent="0.35">
       <c r="A69" s="16" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B69" s="16" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C69" s="16" t="s">
         <v>20</v>
@@ -4398,10 +4444,10 @@
         <v>14</v>
       </c>
       <c r="H69" s="17" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="I69" s="18" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="J69" s="19" t="b">
         <v>0</v>
@@ -4412,7 +4458,7 @@
     </row>
     <row r="70" spans="1:11" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A70" s="16" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B70" s="16" t="s">
         <v>10</v>
@@ -4431,10 +4477,10 @@
         <v>14</v>
       </c>
       <c r="H70" s="16" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="I70" s="17" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="J70" s="19" t="b">
         <v>0</v>
@@ -4445,10 +4491,10 @@
     </row>
     <row r="71" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A71" s="16" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B71" s="16" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C71" s="16" t="s">
         <v>20</v>
@@ -4464,10 +4510,10 @@
         <v>14</v>
       </c>
       <c r="H71" s="17" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="I71" s="18" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="J71" s="19" t="b">
         <v>0</v>
@@ -4478,10 +4524,10 @@
     </row>
     <row r="72" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A72" s="16" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B72" s="16" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C72" s="16" t="s">
         <v>20</v>
@@ -4497,10 +4543,10 @@
         <v>14</v>
       </c>
       <c r="H72" s="17" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="I72" s="18" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="J72" s="19" t="b">
         <v>0</v>
@@ -4511,10 +4557,10 @@
     </row>
     <row r="73" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A73" s="16" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B73" s="16" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C73" s="16" t="s">
         <v>20</v>
@@ -4530,10 +4576,10 @@
         <v>14</v>
       </c>
       <c r="H73" s="17" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="I73" s="18" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="J73" s="19" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
actualización franja horaria colombia
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0526577688ca4eec/Escritorio/Proyectos developer/Diseños_Gasper/Back-end/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1082" documentId="8_{ADBBDD1F-37F2-455A-919D-03174E12E1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD197DE3-9C6B-4378-9E80-462B24D23981}"/>
+  <xr:revisionPtr revIDLastSave="1224" documentId="8_{ADBBDD1F-37F2-455A-919D-03174E12E1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{475A7107-F44D-4D35-AFB3-5531D56FB622}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="356">
   <si>
     <t>name</t>
   </si>
@@ -247,9 +247,6 @@
     <t xml:space="preserve">	deepink,red,blue,orange,darkred,cyan,royalblue,green,olive</t>
   </si>
   <si>
-    <t>{ "deeppink":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250982/dvmu9dgiwvufb7191usm.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250955/slshdhn4kio9xddrtrmq.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250918/fqhuo4tjpp4yczwzdshf.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250921/ahlr0dgh0r98xw4wqud5.png"],"blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250911/indvbpbsahhllbr2demt.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250914/cx8wavuzsrrfeqgehwan.png"],"orange":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250940/hi9axizusckhejfco5s0.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250943/raziqm5ewrpzzjidxqim.png"],"darkred":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250891/zcfxokfughsvu67yjcdh.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250897/gtzajz8mpqk30anhwnhq.png"],"cyan":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250901/nndijkiq3dplak0kmfwk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250904/wh8ugd1vd4yfscmrb8mr.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250907/onk3n4ptbomthsd5ycfk.png"],"royalblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250924/ur5hr32mcpowkradyc1d.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250928/xhpn1wpn0hhufkbbxbci.png"],"green":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250947/ypiwxkfwgbloipv08r3c.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250951/l9xl1h9afd08rzvpze3v.png"],"olive":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250932/hwq3ugjjcdq3xshspdyf.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250936/ima8bakxaxo6mvsch85s.png"]}</t>
-  </si>
-  <si>
     <t xml:space="preserve">	deepink,orange,blue,yellow,red,black,steelblue,olive</t>
   </si>
   <si>
@@ -407,22 +404,6 @@
   </si>
   <si>
     <t>{"white":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205752/mfwiprr6tvgovwpuue2v.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205755/cnpmodwwbutausd84kzo.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205754/vuzoeqyobfg2u01bmwry.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205752/m1pbnbpak4qv1eurewfs.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205758/yii0fqmgiqr2vcn6jobs.png"]}</t>
-  </si>
-  <si>
-    <r>
-      <t>{"lime":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242437/dmbpdy0o8zo774yg0esp.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242493/phwa4ghsnghxaad8rs0s.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242496/z0ckuych5747dbdjbblh.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242497/mllydvsxp8bsmjxtudpf.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242438/gbxh6ouluwykgpjacnn5.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242440/jbincqszbskytgzid1xr.png"],"yellow":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242442/rjagdaxpyr2ekyatvpnc.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242443/omnxdetafnsovhyqsrrk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242445/tfuorgusbozzg5qangpa.png"],"blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242446/vrqh5h2ds6suivfhxsg9.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242448/arvjdgaypjnno56lfvbk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242450/yzbjosqrehdwxvwhcyfo.png"],"orange":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242452/mzxqsxz8cz3pfkwggyzv.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242454/xburffuwfdwwt6917fav.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242455/qgkevnsapc7o43ad0bq7.png"],"gray":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242460/burfwilllus1qaxskiqw.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242460/yspgkvybbozucaqc9ap1.png</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242462/ngof4yshn3cjaat7tglk.png"],"olive":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242498/c9jctj0oy5awxkw7qhps.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242456/lqgzodgnyvwdgdski6al.png"],"deepink":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242501/dzn9seysibv5yjlylqkz.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242464/lxs8m7ci4bwqqyfbrjz5.png"],"white":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242485/t4lvqrs96uqcbrzscv68.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242488/c7sam295q1wiuiiakyt7.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242489/n1csydhjwtdmhlpf30te.png"],"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242479/ony3dvs6kvxistz3fxic.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242481/mmu22qpkw9rz2ecm79rk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242484/afwxcc8qacktmzbo5pcn.png"],"green":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242473/h5jrcvlasfsfetqinrzi.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242473/dfhfnav2renc5azvzicn.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242474/dcsjwceh9gzre70xl9n7.png"],"aqua":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242466/wxbkzpewkatvhqphl8vc.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242469/zlrfrhmdw24co5sql2xg.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242469/oxccamqqxqe81hbdryqd.png"]}</t>
-    </r>
   </si>
   <si>
     <t>{"steelblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773206521/lgdrcsg1bhg9kh7qjnhs.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773206518/hzeq19gaqctil3pzrsi7.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773206525/u9vdtg7rq4zp8awiwcvk.png"],"orange":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773206510/q3vtqnmiruti86ckrgbu.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773206515/me4zdvq6donb2neznfwx.png"],"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773206507/nrjilgz3harir9vbblte.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773206512/sgr2zgufvyugwtetnfwq.png"]}</t>
@@ -478,9 +459,6 @@
   </si>
   <si>
     <t>{"white":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204338/oejbgfjjrnas7l9peyx2.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204336/k7scng21l4yann7xww1g.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204337/p7rhhrzowr2rwabaf4wq.png"],"blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204340/kjystwsspe4qlwkpttbx.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204343/x0wczvaf4thuo262zk1a.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204342/k6n6vrz51vbfxkp37vxw.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204332/klqdeyjspxstecn1fqng.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204334/pmpnlaeem4it8y8tnxn1.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204335/e8dw9g0qre5ydzlqlatf.png"],"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204328/bvt7ueaexvkdythpanwn.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204329/aofbo59s1uffco8i2wpi.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204330/b8n7glynvblcahn4kh05.png"],"pink":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204325/tjdsejcvcgfgkfquxzjn.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204326/mwrayyzb1rfuvdycyddq.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204327/hn8p4ckn1sozzowpziib.png"],"green":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204322/b16ab0jfz0etyo8jshsw.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204321/ooznuwz1cpqaqu5ownul.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204323/q61r8koxk0fhvecqkrfz.png"],"darkblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204319/fkqlvntrdaq8jt793uhj.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204319/a5ep6vrxclrxq3b0h6lk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204320/vckmbagb1qiehbka8qce.png"],"lime":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204344/io3zcwbwx9oayypdxmuc.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204346/shnjivk8vn0zompx1d0k.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204347/uf0mrbixslbi3i4p13qk.png"],"olive":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204350/nhoe6gys7x7a9tr92gcv.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204351/kmf8fquhpmgnpaudotr8.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204351/tvy8pbmxrxbyttnzajdn.png"],"lawngreen":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204355/nmvtfz8xc6seaah6thgh.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204357/wmeg6mwijy05p1hpu3kh.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204358/g5nsawbiilegcqjkcsuk.png"],"mediumblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204361/y8ykrtunchadolpwmw7a.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204363/toeoq0ot4by8nx7y6dfw.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204366/iy9zgfv11qm7vwguueo3.png"],"skyblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204367/b4delwnliq7h2nijhugw.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204368/rxy7ecs4vyuxbllduanx.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773204370/bvmqdttjroiogb5zsevr.png"]}</t>
-  </si>
-  <si>
-    <t>{"lime":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205288/smm8fjw9rl4bnfqartjf.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205287/xibsxjngkirncuy1yzho.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205357/io2ygjdephs2ufzv133d.png"],"blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205290/r3hm9neakhl3lxyiseju.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205292/jasnol7orezj790psdxv.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205294/tp3zzxyom7kg9g40bnug.png"],"green":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205296/lbmq4786zitdm7sqf2gh.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205300/szighhczcmlvktpwcu0c.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205301/zc9grwxp77zytgruhujb.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205305/ip9ubuw7yzb1loywx9hp.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205303/srdszj6njhkynu6hedrq.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205303/srdszj6njhkynu6hedrq.png"],"darkblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205310/in2uykc5yibqy3ii59yd.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205312/auuktvqrfwlpu4yf5zxq.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205314/p8f8kh4dqcbkefuzbxv1.png"],"orange":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205317/masdfk78uq1h1ocqnxon.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205320/ib4jb51wjac4tnbizgel.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205321/bjwnz5zmham8542llwvl.png"],"turquoise":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205323/ghweohyghfzxnp3autyo.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205326/ztc53cu857yxbfpqp193.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205328/ay9h3tyk1kikgchkgh1r.png"],"gray":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205329/hgsinisspnemzvna56cg.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205332/u7f9tauhwezirlpxvghh.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205335/ryi88h3pmqpwnjvruazi.png"],"darkgreen":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205339/eezvjpd0anxakn1d1eir.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205366/afcwdckametvhcm2vdnk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205339/sj4x0jejmfcckjyjcgff.png"],"skyblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205340/ly5tvmjhv2exoglszokt.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205345/mbswblamqqdllr1hzulb.png"],"peru":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205349/ptzps64butp9eg2kdvn5.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205354/spdvczuhihi0kmjzwygz.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205353/uwy3dpacpekdc1mh1k76.png"]}</t>
   </si>
   <si>
     <t>{"blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246712/gotvnqbl4y3hdyauibw5.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246707/yonflyqalxcl4c9if2bj.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246709/xbj5qrmtoxxcqq5damdg.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246714/thwkb1zhc1xobjfnlkec.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246717/lsxqmrzz8lwomqaaua16.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246719/eq8r76oqa5gnfh9gvln8.png"],"green":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246722/ppj4owyqnlqcuebnxv4t.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246725/zzyif5jcihzmwccgjfkf.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246730/dauki5afyvny7y19x5sp.png"],"lime":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246732/wd38ed0dzdwcjwiwzflh.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246737/swfnbkucmbke4llvpasp.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246739/j9jizettng9z4ufui6mh.png"],"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246745/qjkntjcqnncozqokqdai.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246746/dici1svfsqmtnwbaxh3r.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246812/dkdxyqkjivhmzzyiqh8o.png"],"gray":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246817/snvmvdacyeefzgztoegr.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246819/llsaoy4lp3xuig0mzgkz.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246824/qkhbddvmlcesobq3axsl.png"],"skyblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246828/yjyw5k38esggufh9nxoz.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246832/i4h1qxhsejjbg5xnnamq.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773246835/wwsyptj2wb0253mmnltu.png"]}</t>
@@ -1732,25 +1710,6 @@
     <t>blue,red,black, darkred, royalblue</t>
   </si>
   <si>
-    <t>{ "blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253382/k5shc79l7qjtrz6ci2u8.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662299/g4llyutemrjvlpsyhbjl.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662300/qtwerqw10yv6wxqpb1cl.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662299/scdqmabiuqxkreow7u6c.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662302/wghzvjuaajuwpbfddzvk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253384/fa3gtcxcbbujpmz1q32y.png"],"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662299/ys0v7pwpkcommwyjadtf.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662310/tbrnns244roeseqtkxrr.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253383/dxofsgljvhppxhvxcf9q.png"],"darkred":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253383/uqqd6kygifncoygwvzfk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253382/kiy5vdzzlhglrhntyfpf.png"], "royalblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662300/t7f9xsg5ij4gmjrmoyso.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662304/k5128obkwuopjaualtol.png"]}</t>
-  </si>
-  <si>
-    <r>
-      <t>{"lime":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242437/dmbpdy0o8zo774yg0esp.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242493/phwa4ghsnghxaad8rs0s.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242496/z0ckuych5747dbdjbblh.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242497/mllydvsxp8bsmjxtudpf.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242438/gbxh6ouluwykgpjacnn5.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242440/jbincqszbskytgzid1xr.png"],"yellow":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242442/rjagdaxpyr2ekyatvpnc.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242443/omnxdetafnsovhyqsrrk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242445/tfuorgusbozzg5qangpa.png"],"blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242446/vrqh5h2ds6suivfhxsg9.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242448/arvjdgaypjnno56lfvbk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242450/yzbjosqrehdwxvwhcyfo.png"],"orange":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242452/mzxqsxz8cz3pfkwggyzv.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242454/xburffuwfdwwt6917fav.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242455/qgkevnsapc7o43ad0bq7.png"],"gray":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774664553/ckjrrp0qrdw6vn6yqjmf.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774664554/neg0acxwxh0mhhfynsh6.png</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"],"olive":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242498/c9jctj0oy5awxkw7qhps.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242456/lqgzodgnyvwdgdski6al.png"],"deepink":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242501/dzn9seysibv5yjlylqkz.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242464/lxs8m7ci4bwqqyfbrjz5.png"],"white":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242485/t4lvqrs96uqcbrzscv68.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242488/c7sam295q1wiuiiakyt7.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242489/n1csydhjwtdmhlpf30te.png"],"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242479/ony3dvs6kvxistz3fxic.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242481/mmu22qpkw9rz2ecm79rk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242484/afwxcc8qacktmzbo5pcn.png"],"green":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242473/h5jrcvlasfsfetqinrzi.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242473/dfhfnav2renc5azvzicn.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242474/dcsjwceh9gzre70xl9n7.png"],"aqua":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242466/wxbkzpewkatvhqphl8vc.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242469/zlrfrhmdw24co5sql2xg.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242469/oxccamqqxqe81hbdryqd.png"]}</t>
-    </r>
-  </si>
-  <si>
     <t>Enterizo para Ciclismo</t>
   </si>
   <si>
@@ -1968,52 +1927,6 @@
   </si>
   <si>
     <t>Enterizo para Ciclismo.</t>
-  </si>
-  <si>
-    <t>{
-  "black": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715391/agiednmodeb5yfpahlp1.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715392/tofa7d0ks3nqok7en9j6.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715395/cdbcpgyhms197nffsus0.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715394/jpithdawvqp2tmmz4sbr.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715398/aonotdgo3ttkxg3vxife.png"
-  ],
-  "blue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715399/ga18nxoi4pcosvxkgd6x.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715402/u2jtujngu7yuuqdbfo7r.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715403/q1bwntcbzvnilh5xyumu.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715406/nbo3egml3xzqqkgj2yqk.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715407/zdjxkw4a53r0j2kjn5zi.png"
-  ],
-  "gray": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715412/fpyfapenk9fxym7eewmu.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715410/z4kcqsfgasg1z53yarur.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715414/m23amhh21mpotdp88sjn.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715416/ydmz1uralgltpdeevcbc.png"
-  ],
-  "green": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715418/x2rtdwfrfwecvxs84i7l.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715421/ebbezh68fixgh6o84qli.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715423/a7wjeymergff40uhpykt.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715427/oq9maqfvtwrz5cfpmnnw.png"
-  ],
-  "darkblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715428/espsoggmadkxd6weqeb8.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715429/drdkltcampvjzfzc0ifn.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715434/ufwqg1cmoeslcqafsaw9.png"
-  ],
-  "hotpink": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715436/fn4lbigoobdn5xjbm8jh.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715440/ddhq5u6ubbdbbw1no78m.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715441/vb5pyt9y9flu8fh0f45c.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715447/cksicv1hldfrcxgapuug.png"
-  ],
-  "steelblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715449/zhcwcrbc5dkixpezz70b.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715445/koyfabdm2bhnjhkcamu4.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715453/rrada8pae4w27xmxzimc.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715453/ee4ronykxwaebzdtzx8c.png"
-      ],
-  "purple": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715458/uc7n4i1rqltsbblh1ftl.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715460/on3p22rgtcgnqndozwu3.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715460/on3p22rgtcgnqndozwu3.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715465/xxg2fwuxia77qn9dxqtv.png"
-  ],
-  "skyblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715467/bni8lwrz38khcg0wjqss.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715469/zds8ckdyanvwacjut2if.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715475/i3us2trdde2od7imi4yp.png"
-  ]
-}</t>
   </si>
   <si>
     <t>black,blue,gray,green,darkblue,hotpink,steelblue</t>
@@ -2521,23 +2434,6 @@
   </si>
   <si>
     <t>{
-  "green": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058812/wpybvhkk9ugsy6gnxkkm.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058811/d8lzuacyktsdlepm9qcd.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058811/jdmi9kwuwllmglwhhcbc.png"  ],
-  "red": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058814/buq9q1wtddmrrkg6iakf.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058812/b7emupdqe6witatlqvq4.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058814/mkbq6zncote7su95rhag.png" ],
-  "yellow": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058812/d6j3vnuq23pr3pvlqrrc.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058813/sldsj7nnpogk2gxufpxz.png", " https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058814/dmsndzjcdeiql1crljdb.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058814/etvlgtogg1be4ui79eux.png" ],
-  "blue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058814/pwpefqqs0ay3xfzyqep5.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058815/vfq45emabazi47rx4wd0.png" ],
-  "orange": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058815/esequ0cwic5ues3kyrck.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058817/yikzlztavx3gaci9xpfr.png"],
-  "darkblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058816/bg7eetec0kwqfntlzhdu.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058817/hel3nql1dp0vfvjpieyk.png" ],
-  "olive": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058817/xnmxv2e9memmagybowsd.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058816/s6zbit7x8tejpcfnv3s0.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058817/wqonc9kcviofhs7qiatn.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058818/ht4eo6wpkw58c3zsjttb.png" ]}</t>
-  </si>
-  <si>
-    <t>{
   "blue": [
     "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775059351/ms0pfrg6qexy7pvp2b2d.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775059359/knvhre2v1jzwh6slg2m7.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775059355/hgbv0fwafwvnznmhyojl.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775059363/gsrwyckhl9luqezcaslx.png"  ],
   "darkblue": [
@@ -2592,15 +2488,535 @@
     <t>gray,black,darkblue,olive</t>
   </si>
   <si>
+    <t>Esqueleto en Tela Burda</t>
+  </si>
+  <si>
+    <t>olive,red,gray,crimson,purple,white,black,darkblue,darkgreen,blue</t>
+  </si>
+  <si>
+    <t>{
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155269/de0pp7uo7t4rwrcy9na5.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155273/ka4gk0rcnldhraqdzbjt.png" ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155271/sfmzhsktumxhhiykmyl1.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155277/sptbvii9bdz3mfxmmh5u.png"],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155269/uuxdbe3zyuwqasfswvxp.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155270/pcurilqozy4guyqhrr0n.png" ],
+  "crimson": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155273/ldlwpglhvi9ja5q6nmxv.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155271/y805zyiv6vaivssobjjc.png"],
+  "purple": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155271/fwxxwy7bm2f04pld8gpf.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155277/dokov3qhbtqdpxnwjvbg.png"],
+  "white": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155273/sarg592ljgtrlegxr9dg.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155275/b2b7ywzj4heuodk4kd0w.png" ], "black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155272/flxhhmuujdjpezxmkmqn.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155273/j2qcht36qgzywyshdgjj.png"], "darkblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155272/dscu8zuigconhfyshe6z.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155277/eane79kkqkqetsbzchi5.png"],"darkgreen":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155276/jw0lguqjixqg7ke6adqs.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155275/yzp0sx5ta5dlqsraanw6.png"], "blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155273/lyu53mfn62se2kcebbee.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775155278/oiguw01ughqg2mldahy7.png"]}</t>
+  </si>
+  <si>
+    <t>Conjunto Baicker</t>
+  </si>
+  <si>
+    <t>{
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158910/bqfemdrldelrb5vv7s7h.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158925/okysbbknpxhsxub6mctr.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158913/cj8v7h1il0icgey5tw6i.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158921/syghxqv6xfjjwueepbkd.png" ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158914/qqrsusoyogh2qss4s0ec.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158899/a8gwkfjllecgstudd7k3.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158908/unnoqdfkillvgor1ciub.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158912/mo8pyirjuzat9woipnsx.png"],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158906/klvf37lcsveljtrpv2ky.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158911/lwnr8ej3zk5oecuwedv1.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158904/sumzz8ofqyggr6ppc8f0.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158917/pbqufwwuq7ydtcdf17kd.png" ],
+  "crimson": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158910/s0bgdglskoxld0lcd4b9.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158900/ffcz0shmkborvjpnej91.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158897/pdsrxaqwdn0pca9sytz7.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158908/q8pg8snwlwbrbttcpzzm.png"],
+  "purple": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158897/dw9z0ou5vv2bdsodqiub.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158901/vgoxnbpcqdigubexlgno.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158905/nc0ggeaic6thlw8vf6ki.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158922/aoivbzcf7oykus3fcofn.png"],
+  "white": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158888/txin7lhw1hczv1xuqxli.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158887/kdbl9tymc289uyzuiss9.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158888/xrbsm8ivhriszmgokuyi.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158889/nhfvfrnwobb9f1bb8zlo.png" ], "black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158890/ptpqfainiwqfsxac5lp6.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158891/vukm3jfqq4ejhrzhbzdb.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158926/d7mjjss8uxmfdk6jf5ic.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158893/vbpzm6fdkugn7qog1lcp.png"], "darkblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158892/fnctdf2syv6su6ji0dq9.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158919/hcco7fyk6y9o2q4yhi3m.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158907/y4snteswyqdoelc3v0ko.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158916/eiwterq5vxyrduxwyzs0.png"],"darkgreen":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158899/ryrtyjyqbj7ddofhzbin.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158915/jb4asboucaownuqyv4z1.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158925/okysbbknpxhsxub6mctr.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158923/dlvn22nkbnjxtroryyar.png"], "blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158902/ilhxes69tiijyclldzar.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158928/jg9ttyjltwuq8zl5gkbn.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158921/syghxqv6xfjjwueepbkd.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158918/n3jlvokwmaohwiqnmhgx.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158922/npox0trdbvgwyrlimqa8.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775158903/suojpmygqtfzusyrkh1j.png"]}</t>
+  </si>
+  <si>
+    <t>Camiseta Dama</t>
+  </si>
+  <si>
+    <t>red,green,blue</t>
+  </si>
+  <si>
+    <t>{
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775159919/fnfvrj84oklumcmewxlj.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775159917/qcixu8tbtylkifx7oco7.png"],
+  "green": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775159916/cm4hdwxjr7f2istbkskv.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775159921/p5wmomgof1thgldi8ew1.png"],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775159924/osz4oskycnc1mht1s0ig.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775159918/x560apajnl06u2hbsvdl.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775159920/pfesp6ejczmc9rnodkkk.png" ]}</t>
+  </si>
+  <si>
+    <t>Conjunto Esqueleto+Pantaloneta</t>
+  </si>
+  <si>
+    <t>{
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244394/m0lw2mmjnwkzubnnawdt.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244395/b8r0cobeqs1akga3ncs4.png" ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244393/uzxchvtxbxypuk7g8gb0.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244394/hn7z8d0eqzf1zdglzfbn.png"],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244396/uxlcu7efqzqzqjvygtlm.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244395/qioevzt73er4u4wygd7h.png" ],
+  "crimson": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244395/ggmrt6q9supmc1twty5f.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244396/gsmkakv8eh2c5kt9onq7.png"],
+  "purple": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244397/usdxd7zbntng5eunzqce.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244397/jjdhzlbyv3pjqibm8bnl.png"],
+  "white": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244397/lmewpapkk3yqjsagu9lj.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244396/h67pjz4epcgahkndfmg0.png" ], "black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244399/hljbavtshkwprodqxbpc.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244398/mnpxnp2fo9l1goot4ni4.png"], "darkblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244398/suq0rp40vj6ypzfvvjgb.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244410/eutztd2cwgmy1ttnfpvi.png"], "blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244412/xzu6lrtk6rmmspssdvde.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244410/qyxtqokw0bwqf4aouh9d.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244410/ov9r6no428uzisyopj4y.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244411/py1iq21blxizcyungzy3.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244411/uufydwggwngrrecy6pk4.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775244411/xcagxfzz1uquo6labld0.png"]}</t>
+  </si>
+  <si>
+    <t>Conjunto Jogger+Chaqueta Algodón</t>
+  </si>
+  <si>
+    <t>olive,red,gray,crimson,purple,white</t>
+  </si>
+  <si>
+    <t>Conjunto Jogger+Esqueleto</t>
+  </si>
+  <si>
+    <t>{
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188918/gwsz251dgpsj1hew0oya.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188916/blubovl0lekvda8wz28m.png" ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188913/ddpvqzyduogcjuw1fwnn.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188913/l1mde2lin9bwxxd4su3m.png"],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188914/ogdotcnkkdv8rfzbse3i.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188914/mj2tdabjjxpdcr65awvm.png" ],
+  "crimson": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188916/y1qw6mknpnhqwdvbamuq.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188915/kkpxlded8hkqkp5wofp1.png"],
+  "purple": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188915/kq5lpwtcrzbnnubmh54y.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188915/njinwwsp8q6dpnmrwtfg.png"],
+  "white": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188917/vkukktckpia1d7issavr.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188916/xsvvbtlifwxr6wnptmrp.png" ], "black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188918/rybfs9fg7wcmiicwprrv.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188918/kmwubgf9nz3ocioc5qfn.png"], "darkblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188919/n40kc2secr3lstdyyjh1.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775188920/kxlkdyalzfnri32qe0ox.png"]}</t>
+  </si>
+  <si>
+    <t>{
+  "lime": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205288/smm8fjw9rl4bnfqartjf.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205287/xibsxjngkirncuy1yzho.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205357/io2ygjdephs2ufzv133d.png"
+  ],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205290/r3hm9neakhl3lxyiseju.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205292/jasnol7orezj790psdxv.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205294/tp3zzxyom7kg9g40bnug.png"
+  ],
+  "green": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205296/lbmq4786zitdm7sqf2gh.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205300/szighhczcmlvktpwcu0c.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205301/zc9grwxp77zytgruhujb.png"
+  ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205305/ip9ubuw7yzb1loywx9hp.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205303/srdszj6njhkynu6hedrq.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205308/byyt2ryop0d8dr46xt9o.png"
+  ],
+  "darkblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205310/in2uykc5yibqy3ii59yd.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205312/auuktvqrfwlpu4yf5zxq.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205314/p8f8kh4dqcbkefuzbxv1.png"
+  ],
+  "orange": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205317/masdfk78uq1h1ocqnxon.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205320/ib4jb51wjac4tnbizgel.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205321/bjwnz5zmham8542llwvl.png"
+  ],
+  "turquoise": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205323/ghweohyghfzxnp3autyo.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205326/ztc53cu857yxbfpqp193.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205328/ay9h3tyk1kikgchkgh1r.png"
+  ],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205329/hgsinisspnemzvna56cg.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205332/u7f9tauhwezirlpxvghh.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205335/ryi88h3pmqpwnjvruazi.png"
+  ],
+  "darkgreen": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205339/eezvjpd0anxakn1d1eir.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205366/afcwdckametvhcm2vdnk.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205339/sj4x0jejmfcckjyjcgff.png"
+  ],
+  "skyblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205340/ly5tvmjhv2exoglszokt.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205345/mbswblamqqdllr1hzulb.png"
+  ],
+  "peru": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205349/ptzps64butp9eg2kdvn5.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205354/spdvczuhihi0kmjzwygz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773205353/uwy3dpacpekdc1mh1k76.png"
+  ]
+}</t>
+  </si>
+  <si>
     <t>{
   "gray": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080255/czlfuvutd72atp0ojhqh.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080247/xpw55vkz1revjayfz3zz.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080238/itypiaz7qmh7ralcuari.png" ],
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080255/czlfuvutd72atp0ojhqh.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080247/xpw55vkz1revjayfz3zz.png" ],
   "black": [
     "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080241/h3g6polr1fdcf8ygdklb.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080252/yzndprsrmahdoeruuzlt.png" ],
   "darkblue": [
     "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080244/mlvuk1yzzwhccuyxm6hn.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080250/xigvnqz7go87woirjlvb.png" ],
   "olive": [
     "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080236/pxianovllar2lhhacceh.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775080258/jravrpw6pis8ehszhslp.png" ]}</t>
+  </si>
+  <si>
+    <t>{
+  "green": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058812/wpybvhkk9ugsy6gnxkkm.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058811/d8lzuacyktsdlepm9qcd.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058811/jdmi9kwuwllmglwhhcbc.png"  ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058812/b7emupdqe6witatlqvq4.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058814/mkbq6zncote7su95rhag.png" ],
+  "yellow": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058812/d6j3vnuq23pr3pvlqrrc.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058813/sldsj7nnpogk2gxufpxz.png", " https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058814/dmsndzjcdeiql1crljdb.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775267134/mjsaav0j45wdiagbpw6b.png" ],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058814/pwpefqqs0ay3xfzyqep5.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058815/vfq45emabazi47rx4wd0.png" ],
+  "orange": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058815/esequ0cwic5ues3kyrck.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058817/yikzlztavx3gaci9xpfr.png"],
+  "darkblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058816/bg7eetec0kwqfntlzhdu.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058817/hel3nql1dp0vfvjpieyk.png" ],
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058817/xnmxv2e9memmagybowsd.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058816/s6zbit7x8tejpcfnv3s0.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058817/wqonc9kcviofhs7qiatn.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058818/ht4eo6wpkw58c3zsjttb.png" ]}</t>
+  </si>
+  <si>
+    <t>{ "blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253382/k5shc79l7qjtrz6ci2u8.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662299/g4llyutemrjvlpsyhbjl.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662300/qtwerqw10yv6wxqpb1cl.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775267794/oq0hzp8xiepkigd8hytz.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662302/wghzvjuaajuwpbfddzvk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253384/fa3gtcxcbbujpmz1q32y.png"],"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662299/ys0v7pwpkcommwyjadtf.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662310/tbrnns244roeseqtkxrr.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253383/dxofsgljvhppxhvxcf9q.png"],"darkred":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253383/uqqd6kygifncoygwvzfk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253382/kiy5vdzzlhglrhntyfpf.png"], "royalblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662300/t7f9xsg5ij4gmjrmoyso.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662304/k5128obkwuopjaualtol.png"]}</t>
+  </si>
+  <si>
+    <t>{
+  "black": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715391/agiednmodeb5yfpahlp1.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715392/tofa7d0ks3nqok7en9j6.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715395/cdbcpgyhms197nffsus0.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715394/jpithdawvqp2tmmz4sbr.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715398/aonotdgo3ttkxg3vxife.png"
+  ],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715399/ga18nxoi4pcosvxkgd6x.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715402/u2jtujngu7yuuqdbfo7r.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715403/q1bwntcbzvnilh5xyumu.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715406/nbo3egml3xzqqkgj2yqk.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715407/zdjxkw4a53r0j2kjn5zi.png"
+  ],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715412/fpyfapenk9fxym7eewmu.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715410/z4kcqsfgasg1z53yarur.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715414/m23amhh21mpotdp88sjn.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715416/ydmz1uralgltpdeevcbc.png"
+  ],
+  "green": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715418/x2rtdwfrfwecvxs84i7l.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715421/ebbezh68fixgh6o84qli.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715423/a7wjeymergff40uhpykt.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715427/oq9maqfvtwrz5cfpmnnw.png"
+  ],
+  "darkblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715428/espsoggmadkxd6weqeb8.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715429/drdkltcampvjzfzc0ifn.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715434/ufwqg1cmoeslcqafsaw9.png"
+  ],
+  "hotpink": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715436/fn4lbigoobdn5xjbm8jh.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715440/ddhq5u6ubbdbbw1no78m.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715441/vb5pyt9y9flu8fh0f45c.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715447/cksicv1hldfrcxgapuug.png"
+  ],
+  "steelblue": [
+   "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715445/koyfabdm2bhnjhkcamu4.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715453/rrada8pae4w27xmxzimc.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715453/ee4ronykxwaebzdtzx8c.png"
+      ],
+  "purple": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715458/uc7n4i1rqltsbblh1ftl.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715460/on3p22rgtcgnqndozwu3.png",  "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715465/xxg2fwuxia77qn9dxqtv.png"
+  ],
+  "skyblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715467/bni8lwrz38khcg0wjqss.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715469/zds8ckdyanvwacjut2if.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715475/i3us2trdde2od7imi4yp.png"
+  ]
+}</t>
+  </si>
+  <si>
+    <t>{
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189074/gizojaz37bkgea5euugi.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189074/wo3zqlyxwleaxljrpqgm.png" ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189075/mb7ijcwbyzhvmzawc4xc.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189074/fckvvtdkspk6hunvwqcp.png"],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189076/uu44dr65piwmneepq9rb.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189076/mciathn6oxa4yn9rb39w.png" ],
+  "crimson": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189077/zymwn2nrvphztcctx0t0.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189076/lko4bl0upfxl6bpbwcem.png"],
+  "purple": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189078/a1wayfl41mw4zuhlqdrv.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189078/ns2ivpdujrzoqasx3y3p.png"],
+  "white": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189080/w1yav2h8ahdxk9vzel5s.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775189078/ilfiofrwu6y4huewkksx.png" ]}</t>
+  </si>
+  <si>
+    <t>{
+  "lime": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242437/dmbpdy0o8zo774yg0esp.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242493/phwa4ghsnghxaad8rs0s.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242496/z0ckuych5747dbdjbblh.png"
+  ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242497/mllydvsxp8bsmjxtudpf.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242438/gbxh6ouluwykgpjacnn5.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242440/jbincqszbskytgzid1xr.png"
+  ],
+  "yellow": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775270172/c3g6aegbowyrofjqwwyy.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242443/omnxdetafnsovhyqsrrk.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242445/tfuorgusbozzg5qangpa.png"
+  ],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242446/vrqh5h2ds6suivfhxsg9.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242448/arvjdgaypjnno56lfvbk.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242450/yzbjosqrehdwxvwhcyfo.png"
+  ],
+  "orange": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242452/mzxqsxz8cz3pfkwggyzv.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242454/xburffuwfdwwt6917fav.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242455/qgkevnsapc7o43ad0bq7.png"
+  ],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774664553/ckjrrp0qrdw6vn6yqjmf.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774664554/neg0acxwxh0mhhfynsh6.png"
+  ],
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242498/c9jctj0oy5awxkw7qhps.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242456/lqgzodgnyvwdgdski6al.png"
+  ],
+  "deepink": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242501/dzn9seysibv5yjlylqkz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242464/lxs8m7ci4bwqqyfbrjz5.png"
+  ],
+  "white": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242485/t4lvqrs96uqcbrzscv68.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242488/c7sam295q1wiuiiakyt7.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242489/n1csydhjwtdmhlpf30te.png"
+  ],
+  "black": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242479/ony3dvs6kvxistz3fxic.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242481/mmu22qpkw9rz2ecm79rk.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242484/afwxcc8qacktmzbo5pcn.png"
+  ],
+  "green": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242473/h5jrcvlasfsfetqinrzi.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242473/dfhfnav2renc5azvzicn.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242474/dcsjwceh9gzre70xl9n7.png"
+  ],
+  "aqua": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242466/wxbkzpewkatvhqphl8vc.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242469/zlrfrhmdw24co5sql2xg.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242469/oxccamqqxqe81hbdryqd.png"
+  ]
+}</t>
+  </si>
+  <si>
+    <t>blue,red,yellow,lime,orange,gray,olive,deepink,white,black,green,aqua</t>
+  </si>
+  <si>
+    <t>{
+"blue": [
+   "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242450/yzbjosqrehdwxvwhcyfo.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242448/arvjdgaypjnno56lfvbk.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242446/vrqh5h2ds6suivfhxsg9.png"  ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242497/mllydvsxp8bsmjxtudpf.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242438/gbxh6ouluwykgpjacnn5.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242440/jbincqszbskytgzid1xr.png"
+  ],
+  "yellow": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775270172/c3g6aegbowyrofjqwwyy.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242443/omnxdetafnsovhyqsrrk.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242445/tfuorgusbozzg5qangpa.png"
+  ],
+ "lime": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242437/dmbpdy0o8zo774yg0esp.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242493/phwa4ghsnghxaad8rs0s.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242496/z0ckuych5747dbdjbblh.png"  ],
+  "orange": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242452/mzxqsxz8cz3pfkwggyzv.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242454/xburffuwfdwwt6917fav.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242455/qgkevnsapc7o43ad0bq7.png"
+  ],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774664553/ckjrrp0qrdw6vn6yqjmf.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774664554/neg0acxwxh0mhhfynsh6.png"
+  ],
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242498/c9jctj0oy5awxkw7qhps.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242456/lqgzodgnyvwdgdski6al.png"
+  ],
+  "deepink": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242501/dzn9seysibv5yjlylqkz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242464/lxs8m7ci4bwqqyfbrjz5.png"
+  ],
+  "white": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242485/t4lvqrs96uqcbrzscv68.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242488/c7sam295q1wiuiiakyt7.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242489/n1csydhjwtdmhlpf30te.png"
+  ],
+  "black": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242479/ony3dvs6kvxistz3fxic.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242481/mmu22qpkw9rz2ecm79rk.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242484/afwxcc8qacktmzbo5pcn.png"
+  ],
+  "green": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242473/h5jrcvlasfsfetqinrzi.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242473/dfhfnav2renc5azvzicn.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242474/dcsjwceh9gzre70xl9n7.png"
+  ],
+  "aqua": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242466/wxbkzpewkatvhqphl8vc.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242469/zlrfrhmdw24co5sql2xg.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773242469/oxccamqqxqe81hbdryqd.png"
+  ]
+}</t>
+  </si>
+  <si>
+    <t>{
+  "deeppink": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775272048/seolatvo5ibeptxp0qph.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250947/ypiwxkfwgbloipv08r3c.png"
+  ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250921/ahlr0dgh0r98xw4wqud5.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250918/fqhuo4tjpp4yczwzdshf.png"
+  ],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775272044/kzue8vfokuxiyls8okxw.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250911/indvbpbsahhllbr2demt.png"
+  ],
+  "orange": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250943/raziqm5ewrpzzjidxqim.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250940/hi9axizusckhejfco5s0.png"
+  ],
+  "darkred": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775272045/ntqkfjp3ulurkxy4ygdt.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250891/zcfxokfughsvu67yjcdh.png"
+  ],
+  "cyan": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250907/onk3n4ptbomthsd5ycfk.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250901/nndijkiq3dplak0kmfwk.png"
+      ],
+  "royalblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250928/xhpn1wpn0hhufkbbxbci.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250924/ur5hr32mcpowkradyc1d.png"
+  ],
+  "green": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775272044/k0odmztsbytujwkwbj4b.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250932/hwq3ugjjcdq3xshspdyf.png"
+  ],
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250982/dvmu9dgiwvufb7191usm.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773250955/slshdhn4kio9xddrtrmq.png"
+  ]
+}</t>
+  </si>
+  <si>
+    <t>Conjunto Trio</t>
+  </si>
+  <si>
+    <t>{
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530933/uils4eimclbswiqglxwb.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530932/ii7ghf3qbpsqh0hkcx2f.png"
+  ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530933/wjmxysz83faelacafesh.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530933/javfoagq5gzr7uhizidl.png"
+  ],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530935/tx26xvxynmnt13g6jxny.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530937/kxkvlgrfktgso9c0hvwz.png"
+  ],
+  "crimson": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530936/l95akyd4bhk03kowv3yv.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530941/iy0aijqwamomh0fnm5wg.png"
+  ],
+  "purple": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530937/h6rh57doz4ykiom9af59.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530941/rx9im8mi455aitzydnxu.png"
+  ],
+  "white": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530939/twawwnanaibt5slxbfse.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530939/qqz70mll8slv7me5rlku.png"
+  ],
+  "black": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530942/zg4ps6taox8va1al4zug.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530942/b639r0xzf46exnqiqnx1.png"
+  ],
+  "darkblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530934/jjpiskpvm5rsgrpq61an.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530936/cfngz0v2uin3r9pvcnxq.png"
+  ],
+  "darkgreen": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530943/q3xp8jlyr1vds4wnzk9a.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530946/lmuxsq2llfvyfdjout9x.png"
+  ],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530946/itxk54mzlv2ipq17sply.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530944/vo0to0xaxlpifpgzrhde.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775530942/powgxa12h1ygcmpoxuas.png"]
+}</t>
+  </si>
+  <si>
+    <t>{
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528550/gmdzzwnh5cdpqtvymjyv.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528568/tcvv05bz7szpvpwd8zop.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528550/p3hydwhpjpslxexdpanl.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528568/do8kkgmi36vittvqbkiv.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528552/yzfbvjblgnrxzwd29cid.png"
+  ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528552/lvtqga1qb6uwyarixgq6.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528581/dygj9mq5mdrljvnpmrgd.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528552/w6jbg5hjogzaln3jl4j4.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528571/mne0aojjckwvv6fgp5va.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528552/d8xid8l05vqntghit17l.png"
+  ],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528558/kppkvltsc9g6e9skxs60.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528554/zb2b7bs1zohuizr6bhs4.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528617/qjkcgmpyv6z2hrbz0vu9.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528554/ijyksc5bqk511ozo8ych.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528556/z5spj2xo5uvzajchpmqd.png"
+  ],
+  "crimson": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528556/igtbdhfrhc50dar5nhrk.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528567/x2tmdjwsfn85bl3gj2wx.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528658/ztufsmufdck5qppl7xvc.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528557/stin5xulbccessuu2nip.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528557/oqebc4rgn3p6hhafbhtp.png"
+  ],
+  "purple": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528558/msp7kipsfbr6mmzyapzy.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528558/iv8tqyczrfqdk4evrc9i.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528649/hmgwu4h2vjdjta0hwbr3.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528559/t3po7d7m9za9l0dkz994.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528648/arkglftnemydihnmtnlq.png"
+  ],
+  "white": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528559/sjuzzpzilfyiw13k7yes.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528548/aobit1wtczidpesdlq24.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528571/tzuoxfrhjjfssqfrgiym.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528560/fj74tlmoybiupta0nvbr.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528560/lwjlw7wsprqwzppl3yd9.png"
+  ],
+  "black": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528561/rbs2w7fsxdjvmqeb9p2f.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528561/g33p8hylieoiax9n58kr.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528562/jxlvjt6p60as4zefxihn.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528564/e4awddsekmuh4tau6sfj.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528562/zruwjeglcmotxuo76adj.png"
+  ],
+  "darkblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528558/msp7kipsfbr6mmzyapzy.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528546/ilqc1rrwwsfztfcqeuyo.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528546/b8hnh8lbhlwpzvbbh0t3.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528558/kppkvltsc9g6e9skxs60.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528554/cqouzdts64ocfzsl4yof.png"
+  ],
+  "darkgreen": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528546/shatbfwovg3gkyct0jkn.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528568/ljtaegezd3usfkzt2fr3.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528546/qfpysihe3ejliouiacok.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528547/lqhbyrqo4q8ej53scjdh.png"
+  ],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528549/fksujv4reastgqspo0hz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528548/j9yicnf1rr2oncnc1vpi.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528548/aobit1wtczidpesdlq24.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528548/oszx1czsx1bzzf0wdcjq.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775528550/lpfuftrqkjjmufahmofb.png"
+  ]
+}</t>
+  </si>
+  <si>
+    <t>Leggins transparencia Feng Shui</t>
+  </si>
+  <si>
+    <t>Licra de Pecho (Dama).</t>
   </si>
 </sst>
 </file>
@@ -2805,6 +3221,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3092,7 +3512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D9C4F76-C123-4A10-B08E-8C496E2AA870}">
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="57.54296875" style="2" customWidth="1"/>
@@ -3113,7 +3533,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
@@ -3151,10 +3571,10 @@
         <v>16</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>11</v>
@@ -3172,10 +3592,10 @@
         <v>17</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>243</v>
+        <v>344</v>
       </c>
       <c r="K2" s="6" t="b">
         <v>0</v>
@@ -3186,13 +3606,13 @@
     </row>
     <row r="3" spans="1:12" s="3" customFormat="1" ht="99.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>11</v>
@@ -3211,7 +3631,7 @@
         <v>70</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="K3" s="6" t="b">
         <v>0</v>
@@ -3222,13 +3642,13 @@
     </row>
     <row r="4" spans="1:12" s="3" customFormat="1" ht="89.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>11</v>
@@ -3258,15 +3678,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="3" customFormat="1" ht="145" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" s="3" customFormat="1" ht="158.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>20</v>
@@ -3287,7 +3707,7 @@
         <v>73</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>74</v>
+        <v>350</v>
       </c>
       <c r="K5" s="6" t="b">
         <v>0</v>
@@ -3302,7 +3722,7 @@
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>11</v>
@@ -3318,10 +3738,10 @@
         <v>14</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="K6" s="6" t="b">
         <v>0</v>
@@ -3336,7 +3756,7 @@
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>11</v>
@@ -3352,10 +3772,10 @@
         <v>12</v>
       </c>
       <c r="I7" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J7" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>76</v>
       </c>
       <c r="K7" s="6" t="b">
         <v>0</v>
@@ -3370,7 +3790,7 @@
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>11</v>
@@ -3388,10 +3808,10 @@
         <v>13</v>
       </c>
       <c r="I8" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="J8" s="11" t="s">
         <v>77</v>
-      </c>
-      <c r="J8" s="11" t="s">
-        <v>78</v>
       </c>
       <c r="K8" s="6" t="b">
         <v>0</v>
@@ -3402,11 +3822,11 @@
     </row>
     <row r="9" spans="1:12" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>11</v>
@@ -3424,10 +3844,10 @@
         <v>13</v>
       </c>
       <c r="I9" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="J9" s="11" t="s">
         <v>77</v>
-      </c>
-      <c r="J9" s="11" t="s">
-        <v>78</v>
       </c>
       <c r="K9" s="6" t="b">
         <v>0</v>
@@ -3442,7 +3862,7 @@
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>11</v>
@@ -3458,10 +3878,10 @@
         <v>14</v>
       </c>
       <c r="I10" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="J10" s="12" t="s">
         <v>79</v>
-      </c>
-      <c r="J10" s="12" t="s">
-        <v>80</v>
       </c>
       <c r="K10" s="6" t="b">
         <v>0</v>
@@ -3472,11 +3892,11 @@
     </row>
     <row r="11" spans="1:12" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>11</v>
@@ -3492,10 +3912,10 @@
         <v>14</v>
       </c>
       <c r="I11" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="J11" s="12" t="s">
         <v>79</v>
-      </c>
-      <c r="J11" s="12" t="s">
-        <v>80</v>
       </c>
       <c r="K11" s="6" t="b">
         <v>0</v>
@@ -3506,11 +3926,11 @@
     </row>
     <row r="12" spans="1:12" ht="47" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>11</v>
@@ -3525,11 +3945,11 @@
       <c r="H12" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="I12" s="6" t="s">
-        <v>82</v>
+      <c r="I12" s="7" t="s">
+        <v>81</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>128</v>
+        <v>347</v>
       </c>
       <c r="K12" s="6" t="b">
         <v>0</v>
@@ -3540,11 +3960,11 @@
     </row>
     <row r="13" spans="1:12" ht="47" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>11</v>
@@ -3559,11 +3979,11 @@
       <c r="H13" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="I13" s="6" t="s">
-        <v>82</v>
+      <c r="I13" s="7" t="s">
+        <v>348</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>244</v>
+        <v>349</v>
       </c>
       <c r="K13" s="6" t="b">
         <v>0</v>
@@ -3574,11 +3994,11 @@
     </row>
     <row r="14" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>27</v>
@@ -3596,10 +4016,10 @@
         <v>26</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K14" s="6" t="b">
         <v>0</v>
@@ -3610,11 +4030,11 @@
     </row>
     <row r="15" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>27</v>
@@ -3632,10 +4052,10 @@
         <v>26</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K15" s="6" t="b">
         <v>0</v>
@@ -3646,11 +4066,11 @@
     </row>
     <row r="16" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>11</v>
@@ -3668,10 +4088,10 @@
         <v>26</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K16" s="6" t="b">
         <v>0</v>
@@ -3682,11 +4102,11 @@
     </row>
     <row r="17" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>11</v>
@@ -3704,10 +4124,10 @@
         <v>26</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K17" s="6" t="b">
         <v>0</v>
@@ -3722,7 +4142,7 @@
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>30</v>
@@ -3738,10 +4158,10 @@
         <v>28</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K18" s="6" t="b">
         <v>0</v>
@@ -3752,7 +4172,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="6" t="s">
@@ -3772,10 +4192,10 @@
         <v>28</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K19" s="6" t="b">
         <v>0</v>
@@ -3786,11 +4206,11 @@
     </row>
     <row r="20" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>11</v>
@@ -3806,10 +4226,10 @@
         <v>14</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K20" s="6" t="b">
         <v>0</v>
@@ -3824,7 +4244,7 @@
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>11</v>
@@ -3840,10 +4260,10 @@
         <v>14</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J21" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K21" s="6" t="b">
         <v>0</v>
@@ -3858,7 +4278,7 @@
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>11</v>
@@ -3874,10 +4294,10 @@
         <v>32</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J22" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K22" s="6" t="b">
         <v>0</v>
@@ -3892,7 +4312,7 @@
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>11</v>
@@ -3908,10 +4328,10 @@
         <v>14</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J23" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K23" s="6" t="b">
         <v>0</v>
@@ -3926,7 +4346,7 @@
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>11</v>
@@ -3942,10 +4362,10 @@
         <v>14</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J24" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K24" s="6" t="b">
         <v>0</v>
@@ -3960,7 +4380,7 @@
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>11</v>
@@ -3976,10 +4396,10 @@
         <v>14</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="K25" s="6" t="b">
         <v>0</v>
@@ -3990,7 +4410,7 @@
     </row>
     <row r="26" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6" t="s">
@@ -4010,10 +4430,10 @@
         <v>14</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="K26" s="6" t="b">
         <v>0</v>
@@ -4028,7 +4448,7 @@
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>11</v>
@@ -4044,10 +4464,10 @@
         <v>14</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="K27" s="6" t="b">
         <v>0</v>
@@ -4062,7 +4482,7 @@
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>11</v>
@@ -4078,10 +4498,10 @@
         <v>14</v>
       </c>
       <c r="I28" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="J28" s="12" t="s">
         <v>88</v>
-      </c>
-      <c r="J28" s="12" t="s">
-        <v>89</v>
       </c>
       <c r="K28" s="6" t="b">
         <v>0</v>
@@ -4092,7 +4512,7 @@
     </row>
     <row r="29" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="6" t="s">
@@ -4112,10 +4532,10 @@
         <v>41</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J29" s="12" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K29" s="6" t="b">
         <v>0</v>
@@ -4126,7 +4546,7 @@
     </row>
     <row r="30" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="6" t="s">
@@ -4146,10 +4566,10 @@
         <v>41</v>
       </c>
       <c r="I30" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="J30" s="12" t="s">
         <v>91</v>
-      </c>
-      <c r="J30" s="12" t="s">
-        <v>92</v>
       </c>
       <c r="K30" s="6" t="b">
         <v>0</v>
@@ -4182,10 +4602,10 @@
         <v>44</v>
       </c>
       <c r="I31" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J31" s="12" t="s">
         <v>93</v>
-      </c>
-      <c r="J31" s="12" t="s">
-        <v>94</v>
       </c>
       <c r="K31" s="6" t="b">
         <v>0</v>
@@ -4218,10 +4638,10 @@
         <v>45</v>
       </c>
       <c r="I32" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="J32" s="12" t="s">
         <v>95</v>
-      </c>
-      <c r="J32" s="12" t="s">
-        <v>96</v>
       </c>
       <c r="K32" s="6" t="b">
         <v>0</v>
@@ -4252,10 +4672,10 @@
         <v>14</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="K33" s="6" t="b">
         <v>0</v>
@@ -4286,10 +4706,10 @@
         <v>14</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="K34" s="6" t="b">
         <v>0</v>
@@ -4300,7 +4720,7 @@
     </row>
     <row r="35" spans="1:12" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="6" t="s">
@@ -4313,7 +4733,7 @@
         <v>17000</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G35" s="6">
         <v>34000</v>
@@ -4322,10 +4742,10 @@
         <v>41</v>
       </c>
       <c r="I35" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="J35" s="8" t="s">
         <v>98</v>
-      </c>
-      <c r="J35" s="8" t="s">
-        <v>99</v>
       </c>
       <c r="K35" s="6" t="b">
         <v>0</v>
@@ -4336,7 +4756,7 @@
     </row>
     <row r="36" spans="1:12" ht="126.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="6" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="6" t="s">
@@ -4349,7 +4769,7 @@
         <v>17000</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G36" s="6">
         <v>34000</v>
@@ -4358,10 +4778,10 @@
         <v>41</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J36" s="8" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="K36" s="6" t="b">
         <v>0</v>
@@ -4372,7 +4792,7 @@
     </row>
     <row r="37" spans="1:12" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6" t="s">
@@ -4385,7 +4805,7 @@
         <v>17000</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G37" s="6">
         <v>34000</v>
@@ -4394,10 +4814,10 @@
         <v>41</v>
       </c>
       <c r="I37" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J37" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="K37" s="6" t="b">
         <v>0</v>
@@ -4408,7 +4828,7 @@
     </row>
     <row r="38" spans="1:12" ht="91" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="6" t="s">
@@ -4421,7 +4841,7 @@
         <v>17000</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G38" s="6">
         <v>34000</v>
@@ -4430,10 +4850,10 @@
         <v>41</v>
       </c>
       <c r="I38" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="J38" s="8" t="s">
         <v>102</v>
-      </c>
-      <c r="J38" s="8" t="s">
-        <v>103</v>
       </c>
       <c r="K38" s="6" t="b">
         <v>0</v>
@@ -4444,7 +4864,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="6" t="s">
@@ -4464,10 +4884,10 @@
         <v>52</v>
       </c>
       <c r="I39" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="J39" s="12" t="s">
         <v>104</v>
-      </c>
-      <c r="J39" s="12" t="s">
-        <v>105</v>
       </c>
       <c r="K39" s="6" t="b">
         <v>0</v>
@@ -4498,10 +4918,10 @@
         <v>52</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J40" s="13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K40" s="6" t="b">
         <v>0</v>
@@ -4532,10 +4952,10 @@
         <v>14</v>
       </c>
       <c r="I41" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="J41" s="14" t="s">
         <v>107</v>
-      </c>
-      <c r="J41" s="14" t="s">
-        <v>108</v>
       </c>
       <c r="K41" s="6" t="b">
         <v>0</v>
@@ -4546,7 +4966,7 @@
     </row>
     <row r="42" spans="1:12" ht="98.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="6" t="s">
@@ -4566,10 +4986,10 @@
         <v>45</v>
       </c>
       <c r="I42" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J42" s="15" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="K42" s="6" t="b">
         <v>0</v>
@@ -4600,10 +5020,10 @@
         <v>45</v>
       </c>
       <c r="I43" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="J43" s="15" t="s">
         <v>110</v>
-      </c>
-      <c r="J43" s="15" t="s">
-        <v>111</v>
       </c>
       <c r="K43" s="6" t="b">
         <v>0</v>
@@ -4634,10 +5054,10 @@
         <v>14</v>
       </c>
       <c r="I44" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="J44" s="8" t="s">
         <v>300</v>
-      </c>
-      <c r="J44" s="8" t="s">
-        <v>306</v>
       </c>
       <c r="K44" s="6" t="b">
         <v>0</v>
@@ -4670,10 +5090,10 @@
         <v>56</v>
       </c>
       <c r="I45" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="J45" s="8" t="s">
         <v>112</v>
-      </c>
-      <c r="J45" s="8" t="s">
-        <v>113</v>
       </c>
       <c r="K45" s="6" t="b">
         <v>0</v>
@@ -4704,10 +5124,10 @@
         <v>59</v>
       </c>
       <c r="I46" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="J46" s="8" t="s">
         <v>114</v>
-      </c>
-      <c r="J46" s="8" t="s">
-        <v>115</v>
       </c>
       <c r="K46" s="6" t="b">
         <v>0</v>
@@ -4738,10 +5158,10 @@
         <v>13</v>
       </c>
       <c r="I47" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J47" s="15" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K47" s="6" t="b">
         <v>0</v>
@@ -4752,7 +5172,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" s="6" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="6" t="s">
@@ -4772,10 +5192,10 @@
         <v>61</v>
       </c>
       <c r="I48" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="J48" s="14" t="s">
         <v>117</v>
-      </c>
-      <c r="J48" s="14" t="s">
-        <v>118</v>
       </c>
       <c r="K48" s="6" t="b">
         <v>0</v>
@@ -4806,10 +5226,10 @@
         <v>12</v>
       </c>
       <c r="I49" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J49" s="8" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K49" s="6" t="b">
         <v>0</v>
@@ -4824,7 +5244,7 @@
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>11</v>
@@ -4840,10 +5260,10 @@
         <v>12</v>
       </c>
       <c r="I50" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="J50" s="14" t="s">
         <v>120</v>
-      </c>
-      <c r="J50" s="14" t="s">
-        <v>121</v>
       </c>
       <c r="K50" s="6" t="b">
         <v>0</v>
@@ -4874,10 +5294,10 @@
         <v>12</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="J51" s="8" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="K51" s="6" t="b">
         <v>0</v>
@@ -4908,10 +5328,10 @@
         <v>14</v>
       </c>
       <c r="I52" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J52" s="15" t="s">
-        <v>143</v>
+        <v>341</v>
       </c>
       <c r="K52" s="6" t="b">
         <v>0</v>
@@ -4926,7 +5346,7 @@
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>11</v>
@@ -4942,10 +5362,10 @@
         <v>14</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J53" s="12" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="K53" s="6" t="b">
         <v>0</v>
@@ -4960,7 +5380,7 @@
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="6" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D54" s="6" t="s">
         <v>11</v>
@@ -4976,10 +5396,10 @@
         <v>14</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="K54" s="6" t="b">
         <v>0</v>
@@ -4994,7 +5414,7 @@
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>11</v>
@@ -5010,10 +5430,10 @@
         <v>14</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="K55" s="6" t="b">
         <v>0</v>
@@ -5028,7 +5448,7 @@
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D56" s="6" t="s">
         <v>11</v>
@@ -5044,10 +5464,10 @@
         <v>32</v>
       </c>
       <c r="I56" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J56" s="6" t="s">
         <v>126</v>
-      </c>
-      <c r="J56" s="6" t="s">
-        <v>127</v>
       </c>
       <c r="K56" s="6" t="b">
         <v>0</v>
@@ -5058,11 +5478,11 @@
     </row>
     <row r="57" spans="1:12" ht="377" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>11</v>
@@ -5071,7 +5491,7 @@
         <v>22000</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G57" s="6">
         <v>27000</v>
@@ -5080,10 +5500,10 @@
         <v>17</v>
       </c>
       <c r="I57" s="7" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J57" s="15" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="K57" s="6" t="b">
         <v>0</v>
@@ -5094,11 +5514,11 @@
     </row>
     <row r="58" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A58" s="16" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B58" s="16"/>
       <c r="C58" s="16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D58" s="16" t="s">
         <v>27</v>
@@ -5114,10 +5534,10 @@
         <v>14</v>
       </c>
       <c r="I58" s="17" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="J58" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="K58" s="19" t="b">
         <v>0</v>
@@ -5128,11 +5548,11 @@
     </row>
     <row r="59" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A59" s="16" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B59" s="16"/>
       <c r="C59" s="16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D59" s="16" t="s">
         <v>20</v>
@@ -5148,10 +5568,10 @@
         <v>14</v>
       </c>
       <c r="I59" s="17" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="J59" s="18" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="K59" s="19" t="b">
         <v>0</v>
@@ -5162,11 +5582,11 @@
     </row>
     <row r="60" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A60" s="16" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B60" s="16"/>
       <c r="C60" s="16" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D60" s="16" t="s">
         <v>20</v>
@@ -5182,10 +5602,10 @@
         <v>14</v>
       </c>
       <c r="I60" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="J60" s="18" t="s">
         <v>181</v>
-      </c>
-      <c r="J60" s="18" t="s">
-        <v>184</v>
       </c>
       <c r="K60" s="19" t="b">
         <v>0</v>
@@ -5196,11 +5616,11 @@
     </row>
     <row r="61" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A61" s="16" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B61" s="16"/>
       <c r="C61" s="16" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D61" s="16" t="s">
         <v>20</v>
@@ -5216,10 +5636,10 @@
         <v>14</v>
       </c>
       <c r="I61" s="17" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="J61" s="18" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="K61" s="19" t="b">
         <v>0</v>
@@ -5230,11 +5650,11 @@
     </row>
     <row r="62" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A62" s="16" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="16" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D62" s="16" t="s">
         <v>20</v>
@@ -5250,10 +5670,10 @@
         <v>14</v>
       </c>
       <c r="I62" s="17" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="J62" s="18" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="K62" s="19" t="b">
         <v>0</v>
@@ -5264,11 +5684,11 @@
     </row>
     <row r="63" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A63" s="16" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B63" s="16"/>
       <c r="C63" s="16" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D63" s="16" t="s">
         <v>20</v>
@@ -5284,10 +5704,10 @@
         <v>14</v>
       </c>
       <c r="I63" s="17" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="J63" s="18" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="K63" s="19" t="b">
         <v>0</v>
@@ -5298,11 +5718,11 @@
     </row>
     <row r="64" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A64" s="16" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B64" s="16"/>
       <c r="C64" s="16" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D64" s="16" t="s">
         <v>20</v>
@@ -5318,10 +5738,10 @@
         <v>14</v>
       </c>
       <c r="I64" s="17" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="J64" s="18" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="K64" s="19" t="b">
         <v>0</v>
@@ -5332,11 +5752,11 @@
     </row>
     <row r="65" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A65" s="16" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B65" s="16"/>
       <c r="C65" s="16" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D65" s="16" t="s">
         <v>20</v>
@@ -5352,10 +5772,10 @@
         <v>14</v>
       </c>
       <c r="I65" s="17" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="J65" s="18" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="K65" s="19" t="b">
         <v>0</v>
@@ -5366,11 +5786,11 @@
     </row>
     <row r="66" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A66" s="16" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B66" s="16"/>
       <c r="C66" s="16" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D66" s="16" t="s">
         <v>20</v>
@@ -5386,10 +5806,10 @@
         <v>14</v>
       </c>
       <c r="I66" s="17" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="J66" s="18" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="K66" s="19" t="b">
         <v>0</v>
@@ -5400,11 +5820,11 @@
     </row>
     <row r="67" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A67" s="16" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B67" s="16"/>
       <c r="C67" s="16" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D67" s="16" t="s">
         <v>20</v>
@@ -5420,10 +5840,10 @@
         <v>14</v>
       </c>
       <c r="I67" s="17" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="J67" s="18" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="K67" s="19" t="b">
         <v>0</v>
@@ -5434,11 +5854,11 @@
     </row>
     <row r="68" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A68" s="16" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B68" s="16"/>
       <c r="C68" s="16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D68" s="16" t="s">
         <v>20</v>
@@ -5454,10 +5874,10 @@
         <v>14</v>
       </c>
       <c r="I68" s="17" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="J68" s="18" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="K68" s="19" t="b">
         <v>0</v>
@@ -5468,11 +5888,11 @@
     </row>
     <row r="69" spans="1:12" ht="406" x14ac:dyDescent="0.35">
       <c r="A69" s="16" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B69" s="16"/>
       <c r="C69" s="16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D69" s="16" t="s">
         <v>20</v>
@@ -5488,10 +5908,10 @@
         <v>14</v>
       </c>
       <c r="I69" s="17" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="J69" s="18" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="K69" s="19" t="b">
         <v>0</v>
@@ -5502,11 +5922,11 @@
     </row>
     <row r="70" spans="1:12" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A70" s="16" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B70" s="16"/>
       <c r="C70" s="16" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="D70" s="16" t="s">
         <v>20</v>
@@ -5522,10 +5942,10 @@
         <v>14</v>
       </c>
       <c r="I70" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="J70" s="17" t="s">
         <v>213</v>
-      </c>
-      <c r="J70" s="17" t="s">
-        <v>216</v>
       </c>
       <c r="K70" s="19" t="b">
         <v>0</v>
@@ -5536,11 +5956,11 @@
     </row>
     <row r="71" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A71" s="16" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B71" s="16"/>
       <c r="C71" s="16" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D71" s="16" t="s">
         <v>20</v>
@@ -5556,10 +5976,10 @@
         <v>14</v>
       </c>
       <c r="I71" s="17" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="J71" s="18" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="K71" s="19" t="b">
         <v>0</v>
@@ -5570,11 +5990,11 @@
     </row>
     <row r="72" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A72" s="16" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B72" s="16"/>
       <c r="C72" s="16" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D72" s="16" t="s">
         <v>20</v>
@@ -5590,10 +6010,10 @@
         <v>14</v>
       </c>
       <c r="I72" s="17" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="J72" s="18" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="K72" s="19" t="b">
         <v>0</v>
@@ -5604,11 +6024,11 @@
     </row>
     <row r="73" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A73" s="16" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B73" s="16"/>
       <c r="C73" s="16" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D73" s="16" t="s">
         <v>20</v>
@@ -5624,10 +6044,10 @@
         <v>14</v>
       </c>
       <c r="I73" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="J73" s="18" t="s">
         <v>219</v>
-      </c>
-      <c r="J73" s="18" t="s">
-        <v>222</v>
       </c>
       <c r="K73" s="19" t="b">
         <v>0</v>
@@ -5638,13 +6058,13 @@
     </row>
     <row r="74" spans="1:12" ht="319" x14ac:dyDescent="0.35">
       <c r="A74" s="16" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="B74" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C74" s="16" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="D74" s="16" t="s">
         <v>11</v>
@@ -5657,13 +6077,13 @@
         <v>34000</v>
       </c>
       <c r="H74" s="16" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="I74" s="16" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="J74" s="18" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="K74" s="19" t="b">
         <v>0</v>
@@ -5674,11 +6094,11 @@
     </row>
     <row r="75" spans="1:12" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A75" s="16" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B75" s="16"/>
       <c r="C75" s="16" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D75" s="16" t="s">
         <v>20</v>
@@ -5694,10 +6114,10 @@
         <v>14</v>
       </c>
       <c r="I75" s="16" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="J75" s="18" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="K75" s="19" t="b">
         <v>0</v>
@@ -5708,11 +6128,11 @@
     </row>
     <row r="76" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A76" s="16" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B76" s="16"/>
       <c r="C76" s="16" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D76" s="16" t="s">
         <v>20</v>
@@ -5728,10 +6148,10 @@
         <v>14</v>
       </c>
       <c r="I76" s="17" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="J76" s="17" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K76" s="19" t="b">
         <v>0</v>
@@ -5742,11 +6162,11 @@
     </row>
     <row r="77" spans="1:12" ht="87" x14ac:dyDescent="0.35">
       <c r="A77" s="16" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B77" s="16"/>
       <c r="C77" s="16" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D77" s="16" t="s">
         <v>20</v>
@@ -5762,10 +6182,10 @@
         <v>14</v>
       </c>
       <c r="I77" s="16" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="J77" s="18" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="K77" s="19" t="b">
         <v>0</v>
@@ -5776,13 +6196,13 @@
     </row>
     <row r="78" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A78" s="16" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="B78" s="16" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="C78" s="16" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D78" s="16" t="s">
         <v>20</v>
@@ -5798,10 +6218,10 @@
         <v>14</v>
       </c>
       <c r="I78" s="17" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="J78" s="18" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="K78" s="19" t="b">
         <v>0</v>
@@ -5812,13 +6232,13 @@
     </row>
     <row r="79" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A79" s="16" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B79" s="16" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="C79" s="16" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D79" s="16" t="s">
         <v>20</v>
@@ -5834,10 +6254,10 @@
         <v>14</v>
       </c>
       <c r="I79" s="17" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="J79" s="18" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="K79" s="19" t="b">
         <v>0</v>
@@ -5848,11 +6268,11 @@
     </row>
     <row r="80" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A80" s="16" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B80" s="16"/>
       <c r="C80" s="16" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D80" s="16" t="s">
         <v>20</v>
@@ -5868,10 +6288,10 @@
         <v>14</v>
       </c>
       <c r="I80" s="16" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="J80" s="17" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="K80" s="19" t="b">
         <v>0</v>
@@ -5882,11 +6302,11 @@
     </row>
     <row r="81" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A81" s="16" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="B81" s="16"/>
       <c r="C81" s="16" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D81" s="16" t="s">
         <v>20</v>
@@ -5902,10 +6322,10 @@
         <v>14</v>
       </c>
       <c r="I81" s="16" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="J81" s="17" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="K81" s="19" t="b">
         <v>0</v>
@@ -5916,11 +6336,11 @@
     </row>
     <row r="82" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A82" s="16" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="B82" s="16"/>
       <c r="C82" s="16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D82" s="16" t="s">
         <v>20</v>
@@ -5936,10 +6356,10 @@
         <v>14</v>
       </c>
       <c r="I82" s="17" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="J82" s="18" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="K82" s="19" t="b">
         <v>0</v>
@@ -5950,11 +6370,11 @@
     </row>
     <row r="83" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A83" s="16" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B83" s="16"/>
       <c r="C83" s="16" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D83" s="16" t="s">
         <v>20</v>
@@ -5970,10 +6390,10 @@
         <v>14</v>
       </c>
       <c r="I83" s="17" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="J83" s="21" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="K83" s="19" t="b">
         <v>0</v>
@@ -5984,11 +6404,11 @@
     </row>
     <row r="84" spans="1:12" ht="261" x14ac:dyDescent="0.35">
       <c r="A84" s="16" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B84" s="16"/>
       <c r="C84" s="16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D84" s="16" t="s">
         <v>20</v>
@@ -6004,10 +6424,10 @@
         <v>14</v>
       </c>
       <c r="I84" s="16" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="J84" s="21" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="K84" s="19" t="b">
         <v>0</v>
@@ -6018,11 +6438,11 @@
     </row>
     <row r="85" spans="1:12" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A85" s="16" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B85" s="16"/>
       <c r="C85" s="16" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D85" s="16" t="s">
         <v>20</v>
@@ -6031,7 +6451,7 @@
         <v>25000</v>
       </c>
       <c r="F85" s="17" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="G85" s="16">
         <v>36000</v>
@@ -6040,10 +6460,10 @@
         <v>13</v>
       </c>
       <c r="I85" s="16" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="J85" s="21" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="K85" s="19" t="b">
         <v>0</v>
@@ -6054,11 +6474,11 @@
     </row>
     <row r="86" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A86" s="16" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B86" s="16"/>
       <c r="C86" s="16" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D86" s="16" t="s">
         <v>20</v>
@@ -6074,10 +6494,10 @@
         <v>14</v>
       </c>
       <c r="I86" s="17" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="J86" s="21" t="s">
-        <v>271</v>
+        <v>345</v>
       </c>
       <c r="K86" s="19" t="b">
         <v>0</v>
@@ -6088,11 +6508,11 @@
     </row>
     <row r="87" spans="1:12" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A87" s="6" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="6" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D87" s="6" t="s">
         <v>11</v>
@@ -6108,10 +6528,10 @@
         <v>12</v>
       </c>
       <c r="I87" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J87" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="J87" s="11" t="s">
-        <v>76</v>
       </c>
       <c r="K87" s="6" t="b">
         <v>0</v>
@@ -6122,7 +6542,7 @@
     </row>
     <row r="88" spans="1:12" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A88" s="6" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="B88" s="6"/>
       <c r="C88" s="6" t="s">
@@ -6139,13 +6559,13 @@
         <v>27000</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="I88" s="7" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="J88" s="22" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="K88" s="6" t="b">
         <v>0</v>
@@ -6156,7 +6576,7 @@
     </row>
     <row r="89" spans="1:12" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A89" s="6" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="B89" s="6"/>
       <c r="C89" s="6" t="s">
@@ -6176,10 +6596,10 @@
         <v>14</v>
       </c>
       <c r="I89" s="7" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="J89" s="22" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="K89" s="6" t="b">
         <v>0</v>
@@ -6190,11 +6610,11 @@
     </row>
     <row r="90" spans="1:12" ht="319" x14ac:dyDescent="0.35">
       <c r="A90" s="6" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="B90" s="6"/>
       <c r="C90" s="6" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="D90" s="6" t="s">
         <v>11</v>
@@ -6210,10 +6630,10 @@
         <v>12</v>
       </c>
       <c r="I90" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J90" s="8" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K90" s="6" t="b">
         <v>0</v>
@@ -6224,11 +6644,11 @@
     </row>
     <row r="91" spans="1:12" ht="319" x14ac:dyDescent="0.35">
       <c r="A91" s="23" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="B91" s="23"/>
       <c r="C91" s="23" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="D91" s="23" t="s">
         <v>11</v>
@@ -6241,13 +6661,13 @@
         <v>45000</v>
       </c>
       <c r="H91" s="23" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="I91" s="7" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="J91" s="22" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="K91" s="6" t="b">
         <v>0</v>
@@ -6258,7 +6678,7 @@
     </row>
     <row r="92" spans="1:12" ht="391.5" x14ac:dyDescent="0.35">
       <c r="A92" s="23" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="B92" s="23"/>
       <c r="C92" s="23" t="s">
@@ -6278,10 +6698,10 @@
         <v>14</v>
       </c>
       <c r="I92" s="24" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="J92" s="22" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="K92" s="6" t="b">
         <v>0</v>
@@ -6292,11 +6712,11 @@
     </row>
     <row r="93" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A93" s="23" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="B93" s="23"/>
       <c r="C93" s="23" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D93" s="23" t="s">
         <v>20</v>
@@ -6312,10 +6732,10 @@
         <v>14</v>
       </c>
       <c r="I93" s="7" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="J93" s="11" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="K93" s="6" t="b">
         <v>0</v>
@@ -6326,11 +6746,11 @@
     </row>
     <row r="94" spans="1:12" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A94" s="25" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="B94" s="25"/>
       <c r="C94" s="25" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D94" s="25" t="s">
         <v>20</v>
@@ -6346,10 +6766,10 @@
         <v>14</v>
       </c>
       <c r="I94" s="25" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="J94" s="26" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="K94" s="25" t="b">
         <v>0</v>
@@ -6360,11 +6780,11 @@
     </row>
     <row r="95" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A95" s="25" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="B95" s="25"/>
       <c r="C95" s="25" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D95" s="25" t="s">
         <v>20</v>
@@ -6380,10 +6800,10 @@
         <v>61</v>
       </c>
       <c r="I95" s="26" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="J95" s="27" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="K95" s="25" t="b">
         <v>0</v>
@@ -6394,11 +6814,11 @@
     </row>
     <row r="96" spans="1:12" ht="261" x14ac:dyDescent="0.35">
       <c r="A96" s="25" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="B96" s="25"/>
       <c r="C96" s="25" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D96" s="25" t="s">
         <v>20</v>
@@ -6414,10 +6834,10 @@
         <v>14</v>
       </c>
       <c r="I96" s="25" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="J96" s="27" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="K96" s="25" t="b">
         <v>0</v>
@@ -6428,11 +6848,11 @@
     </row>
     <row r="97" spans="1:12" ht="174" x14ac:dyDescent="0.35">
       <c r="A97" s="25" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="B97" s="25"/>
       <c r="C97" s="25" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D97" s="25" t="s">
         <v>20</v>
@@ -6448,10 +6868,10 @@
         <v>14</v>
       </c>
       <c r="I97" s="25" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="J97" s="26" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="K97" s="25" t="b">
         <v>0</v>
@@ -6462,11 +6882,11 @@
     </row>
     <row r="98" spans="1:12" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A98" s="25" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="B98" s="25"/>
       <c r="C98" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D98" s="25" t="s">
         <v>20</v>
@@ -6482,10 +6902,10 @@
         <v>14</v>
       </c>
       <c r="I98" s="26" t="s">
+        <v>314</v>
+      </c>
+      <c r="J98" s="26" t="s">
         <v>320</v>
-      </c>
-      <c r="J98" s="26" t="s">
-        <v>327</v>
       </c>
       <c r="K98" s="25" t="b">
         <v>0</v>
@@ -6496,11 +6916,11 @@
     </row>
     <row r="99" spans="1:12" ht="319" x14ac:dyDescent="0.35">
       <c r="A99" s="25" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="B99" s="25"/>
       <c r="C99" s="25" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D99" s="25" t="s">
         <v>20</v>
@@ -6516,10 +6936,10 @@
         <v>14</v>
       </c>
       <c r="I99" s="26" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="J99" s="26" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="K99" s="25" t="b">
         <v>0</v>
@@ -6530,11 +6950,11 @@
     </row>
     <row r="100" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A100" s="25" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="B100" s="25"/>
       <c r="C100" s="25" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D100" s="25" t="s">
         <v>20</v>
@@ -6550,10 +6970,10 @@
         <v>14</v>
       </c>
       <c r="I100" s="26" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="J100" s="26" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="K100" s="25" t="b">
         <v>0</v>
@@ -6562,13 +6982,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:12" ht="406" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" ht="391.5" x14ac:dyDescent="0.35">
       <c r="A101" s="28" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="B101" s="28"/>
       <c r="C101" s="28" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D101" s="28" t="s">
         <v>20</v>
@@ -6584,10 +7004,10 @@
         <v>14</v>
       </c>
       <c r="I101" s="29" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="J101" s="29" t="s">
-        <v>326</v>
+        <v>343</v>
       </c>
       <c r="K101" s="28" t="b">
         <v>0</v>
@@ -6598,11 +7018,11 @@
     </row>
     <row r="102" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A102" s="25" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="B102" s="25"/>
       <c r="C102" s="25" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D102" s="25" t="s">
         <v>20</v>
@@ -6618,10 +7038,10 @@
         <v>14</v>
       </c>
       <c r="I102" s="26" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="J102" s="26" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="K102" s="25" t="b">
         <v>0</v>
@@ -6630,13 +7050,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:12" ht="203" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A103" s="28" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="B103" s="28"/>
       <c r="C103" s="28" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D103" s="28" t="s">
         <v>11</v>
@@ -6652,15 +7072,321 @@
         <v>14</v>
       </c>
       <c r="I103" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="J103" s="29" t="s">
+        <v>342</v>
+      </c>
+      <c r="K103" s="28" t="b">
+        <v>0</v>
+      </c>
+      <c r="L103" s="28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" ht="391.5" x14ac:dyDescent="0.35">
+      <c r="A104" s="28" t="s">
+        <v>327</v>
+      </c>
+      <c r="B104" s="28"/>
+      <c r="C104" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="D104" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E104" s="28">
+        <v>20000</v>
+      </c>
+      <c r="F104" s="28"/>
+      <c r="G104" s="28">
+        <v>24000</v>
+      </c>
+      <c r="H104" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="I104" s="29" t="s">
+        <v>328</v>
+      </c>
+      <c r="J104" s="29" t="s">
+        <v>329</v>
+      </c>
+      <c r="K104" s="28" t="b">
+        <v>0</v>
+      </c>
+      <c r="L104" s="28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A105" s="25" t="s">
+        <v>330</v>
+      </c>
+      <c r="B105" s="25"/>
+      <c r="C105" s="25" t="s">
+        <v>171</v>
+      </c>
+      <c r="D105" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="E105" s="25">
+        <v>21000</v>
+      </c>
+      <c r="F105" s="25"/>
+      <c r="G105" s="25">
+        <v>31500</v>
+      </c>
+      <c r="H105" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="I105" s="26" t="s">
+        <v>328</v>
+      </c>
+      <c r="J105" s="26" t="s">
+        <v>331</v>
+      </c>
+      <c r="K105" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="L105" s="25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A106" s="25" t="s">
+        <v>332</v>
+      </c>
+      <c r="B106" s="25"/>
+      <c r="C106" s="25" t="s">
+        <v>179</v>
+      </c>
+      <c r="D106" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="E106" s="25">
+        <v>8000</v>
+      </c>
+      <c r="F106" s="25"/>
+      <c r="G106" s="25">
+        <v>12000</v>
+      </c>
+      <c r="H106" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="I106" s="25" t="s">
         <v>333</v>
       </c>
-      <c r="J103" s="29" t="s">
+      <c r="J106" s="26" t="s">
         <v>334</v>
       </c>
-      <c r="K103" s="28" t="b">
-        <v>0</v>
-      </c>
-      <c r="L103" s="28" t="b">
+      <c r="K106" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="L106" s="25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A107" s="28" t="s">
+        <v>335</v>
+      </c>
+      <c r="B107" s="28"/>
+      <c r="C107" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="D107" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E107" s="28">
+        <v>46000</v>
+      </c>
+      <c r="F107" s="28"/>
+      <c r="G107" s="28">
+        <v>68500</v>
+      </c>
+      <c r="H107" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="I107" s="29" t="s">
+        <v>328</v>
+      </c>
+      <c r="J107" s="29" t="s">
+        <v>336</v>
+      </c>
+      <c r="K107" s="28" t="b">
+        <v>0</v>
+      </c>
+      <c r="L107" s="28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" ht="275.5" x14ac:dyDescent="0.35">
+      <c r="A108" s="28" t="s">
+        <v>337</v>
+      </c>
+      <c r="B108" s="28"/>
+      <c r="C108" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="D108" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E108" s="28">
+        <v>68000</v>
+      </c>
+      <c r="F108" s="28"/>
+      <c r="G108" s="28">
+        <v>102000</v>
+      </c>
+      <c r="H108" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="I108" s="28" t="s">
+        <v>338</v>
+      </c>
+      <c r="J108" s="29" t="s">
+        <v>346</v>
+      </c>
+      <c r="K108" s="28" t="b">
+        <v>0</v>
+      </c>
+      <c r="L108" s="28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" ht="333.5" x14ac:dyDescent="0.35">
+      <c r="A109" s="28" t="s">
+        <v>339</v>
+      </c>
+      <c r="B109" s="28"/>
+      <c r="C109" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="D109" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E109" s="28">
+        <v>58000</v>
+      </c>
+      <c r="F109" s="28"/>
+      <c r="G109" s="28">
+        <v>87000</v>
+      </c>
+      <c r="H109" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="I109" s="29" t="s">
+        <v>338</v>
+      </c>
+      <c r="J109" s="29" t="s">
+        <v>340</v>
+      </c>
+      <c r="K109" s="28" t="b">
+        <v>0</v>
+      </c>
+      <c r="L109" s="28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A110" s="25" t="s">
+        <v>351</v>
+      </c>
+      <c r="B110" s="25"/>
+      <c r="C110" s="25" t="s">
+        <v>171</v>
+      </c>
+      <c r="D110" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="E110" s="25">
+        <v>27000</v>
+      </c>
+      <c r="F110" s="25"/>
+      <c r="G110" s="25">
+        <v>40500</v>
+      </c>
+      <c r="H110" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="I110" s="26" t="s">
+        <v>328</v>
+      </c>
+      <c r="J110" s="26" t="s">
+        <v>353</v>
+      </c>
+      <c r="K110" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="L110" s="25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A111" s="25" t="s">
+        <v>354</v>
+      </c>
+      <c r="B111" s="25"/>
+      <c r="C111" s="25" t="s">
+        <v>194</v>
+      </c>
+      <c r="D111" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="E111" s="25">
+        <v>15000</v>
+      </c>
+      <c r="F111" s="25"/>
+      <c r="G111" s="25">
+        <v>22500</v>
+      </c>
+      <c r="H111" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="I111" s="26" t="s">
+        <v>328</v>
+      </c>
+      <c r="J111" s="26" t="s">
+        <v>352</v>
+      </c>
+      <c r="K111" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="L111" s="25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" ht="275.5" x14ac:dyDescent="0.35">
+      <c r="A112" s="25" t="s">
+        <v>355</v>
+      </c>
+      <c r="B112" s="25"/>
+      <c r="C112" s="25" t="s">
+        <v>179</v>
+      </c>
+      <c r="D112" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="E112" s="25">
+        <v>19000</v>
+      </c>
+      <c r="F112" s="25"/>
+      <c r="G112" s="25">
+        <v>19000</v>
+      </c>
+      <c r="H112" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="I112" s="26" t="s">
+        <v>314</v>
+      </c>
+      <c r="J112" s="26" t="s">
+        <v>320</v>
+      </c>
+      <c r="K112" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="L112" s="25" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
actualización recepción de archivos
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0526577688ca4eec/Escritorio/Proyectos developer/Diseños_Gasper/Back-end/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1276" documentId="8_{ADBBDD1F-37F2-455A-919D-03174E12E1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3F27347-06D3-45D9-A37E-364C6C39D771}"/>
+  <xr:revisionPtr revIDLastSave="1301" documentId="8_{ADBBDD1F-37F2-455A-919D-03174E12E1B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4505801C-7DFA-48C9-9E4A-9720EA84FEE9}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="productos" sheetId="2" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="371">
   <si>
     <t>name</t>
   </si>
@@ -179,9 +179,6 @@
   </si>
   <si>
     <t>S,M,L</t>
-  </si>
-  <si>
-    <t>Rompevientos Maya Interna</t>
   </si>
   <si>
     <t>Chaqueta Selección Colombia</t>
@@ -1167,28 +1164,6 @@
     <t>Conjunto Deportivo Buso y Leggins</t>
   </si>
   <si>
-    <t>{
-  "pink": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420046/o4phycvt82wjz8kplszr.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420265/twvchekif2zodyxanc1i.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420049/db3k6djx5iehvdk5tzsb.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420266/s8wejcy8ethxjhvwfim1.png"
-  ],
-  "blue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420039/zy4nsioggmxibakgkmnq.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420258/befqhobvwpandubpdwnx.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420208/nsi9nfrc9iwjh549x27f.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420041/oscbxkl0amqrovmxdl96.png"
-    ],
-  "gray": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420271/emoayd31qpmmzq1e3cow.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420209/grarwuvkojfsxp3zkkea.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420219/iej9eryy6zmsqpxbtren.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420269/ssqsptxxtzk5242meapv.png"
-   ],
-  "green": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420212/dwppw1yttgi1glfoirjp.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420261/tsukkdewe1ssc9fx1xyf.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420213/nslqbwrpsalmznectkju.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420205/tjubdm4z489rrllcpjae.png"
-    ],
-  "darkblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420050/a3sah9k0vso0yczkejjp.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420217/qqxejrn7vafzp7mxinpd.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420203/tjmfayvfgtfwvotp3w7b.png" ],
-  "hotpink": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420202/mllthenng41x09edlbhz.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420045/a2ajlcckgz0jrgzkc5ym.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420259/rpf0na4o552r5leox8lp.png"  ],
-  "steelblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420215/ctwopprmeqldjrqo7ore.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420277/vme2qfi6m8fkbpuuwwmw.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420273/eigh1jdqa5mypkwg9lf9.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420043/hgp1p2lxyof2jxtglg7u.png"
-  ]}</t>
-  </si>
-  <si>
     <t>Conjunto Bicicletero y Top Combinado</t>
   </si>
   <si>
@@ -1207,174 +1182,6 @@
     ],
   "darkblue": [
     "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421319/d9qqgtc0yluoaqb2nhss.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773421294/hniugnmmmcgs8gfc3kyq.png"]}</t>
-  </si>
-  <si>
-    <t>{
-  "pink": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072753/dsppjvpwowbghyyabeog.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072754/iufnbxgh8v2t6nun4m8f.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072791/lycg5baqgojxovlk3klq.png"
-  ],
-  "blue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072764/q9ui9mat04sqcn7jpqb8.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072753/vaefzvoqosvza2tjc04h.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072751/tktrkjoftskg81kjytab.png"
-    ],
-  "gray": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072762/oxepi3ridavl6iaquioe.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072768/jibcdv8zdbbnl2shknx5.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415974/zlvlfegmwgwtj3uegmf6.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072784/lkxruusxffwbja8pvoem.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072794/htikpbl3pq2mpqp2ps8r.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072753/egdi0tylliek1qyjso6x.png"
-   ],
-  "green": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072758/tfir7j2qcftiffz8aca6.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072757/schvcegqk9teituzut2v.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072772/fuhllgv2gcygjv5uvhqx.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072786/iulimynpkmgyp1lrfyca.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072787/fhvdbb22uf43y6a8y3pz.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072763/xjzgglbt4ryzsr1dvjul.png"
-    ],
-  "darkblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072771/ocuhg6y7bx3q4k6qswwm.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072761/to6r3iw5czbnugwicbyo.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072755/njj3ykdg4wphlwueohpp.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072772/smojgyyxywm1ppopmhac.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072766/ehfpqr0onlnnfcmxkw6g.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072765/aijvgan44bsdlarde9hu.png"],
-  "hotpink": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072776/xy0oq8u2z354b9irwdi0.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072760/f7qv7ihynasmahakerzr.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072759/khvijabocbvnua4rq4vt.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072778/mey8d1cqjigzohe2kfsh.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072791/pglujdgbvmqn12el2igs.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072752/lud7tphmwdzz98gq2bkm.png"  ],
-  "steelblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072778/rt8jsbd8g77dtmflde6n.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072783/qzzslyqihjzfteprnqu3.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072756/nrlasih250wtk3djzpne.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072781/ecdvpj1gcs5bf219hskg.png"
-  ]}</t>
-  </si>
-  <si>
-    <t>{
-  "pink": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416290/qrlowbtwfkpfypavclt5.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416053/k746fugxvqwjknpiychz.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416262/wqdfvzcho2lfxta4gzgz.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416311/ooa4txwpixsa1zktiz0o.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416190/nf2325leitsuv0tua7lf.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416250/ets5y8x1rkziuisz27vd.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416286/bn9euxkqhrbqlmvuhxiz.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416207/bmecxkohc2lcciefvprm.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416302/fc0pvuenvqudhe0ry818.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416195/kqzwt4sp5q0ge1hh8dwq.png"
-  ],
-  "blue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416294/pmshoq3tjgafq6gpcbt9.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416273/uogfsfsucmmsnyepdtbb.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416220/jdzz1cc3iaizq4j4dz6e.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416183/filmlgbtdgt2pd2pjeuo.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416323/qmthfapue8mwtsxurtfz.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416244/vxyttjxduexjvje1lvm6.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416215/snrk8fldawf0oirrvquv.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416178/pr4qhmhhxtvt0d5apipa.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415980/gzezgzr4ue2yp3mu5rzo.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416196/f9jdzglnonjv9mrqmrea.png"
-  ],
-  "gray": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415970/j0emdwlkpwvkwyofrxkv.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416208/jksbv56emig4qz94gmu9.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415974/zlvlfegmwgwtj3uegmf6.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416294/gom3hdiys0lpegiucrfa.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416262/hqptcmqk7le05zjivb2k.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416312/tbaamx57e76vf6gpb7wz.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416316/yvchju9wkaf9elfxm2w6.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416263/xdmzoozc7dhxq6cuze6i.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416320/iq8yndysogkwqyeie3t1.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415991/t796xjnfo98lb7bhmvsq.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416310/ohb69dmxvobxucufp8fz.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416289/hycllrw7ygufhch0nysq.png"
-  ],
-  "green": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416166/qrqgdfj7kqlb9zfng6og.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415990/j3al7u3gj7mkaku0qoby.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415980/cnnqftkwrshlexyjlapl.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415959/kjxny6jnzipqvk91ok2x.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415995/na8186pgdaqwniyxhose.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416176/s1w9mmdlhvuqb2avrrad.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415984/dpccybijitpf8ji3iteu.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416285/ybuu7gx8wzf3jejflzts.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416187/vioijghseh9sdqf2nkal.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416300/divgdwrvstqluscll2lf.png"
-  ],
-  "darkblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416299/fpqonbmnz6qfdppdzmsl.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416295/cwxjgbndrpebrw4dya7c.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416272/yutx8qm1vkjeggh99ew7.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416177/gsen39sqfogt42jmlpez.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415973/voeon9pukrdqtvq128kv.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416211/ubqgbda3rjout3urkw09.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416168/se1krtmrlk6epe6mmqzz.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416242/wtlrtruu93kuzt61p55z.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416243/fcuvs7v55a66f46l0jed.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416310/bjypkov8tqc4gvms7tod.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415965/cvx3oyygwzfxfgj3mgof.png"
-  ],
-  "hotpink": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415987/iuyjozzwro18snorgkaz.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416003/vou1uotpawlgvdow6blj.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416228/grpnayzcsu7pwysdpm9l.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416336/so117psdpsxbfxn86aa4.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416212/clo6omrpdsqacmfbyx2e.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416003/nal0y1aousnydel9c9bh.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416167/wh3yinojxhalhz4qe3rg.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416180/yariiiyggalcawpthysm.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416317/eonvxsrpzrhn2vlcjatj.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416203/lv6d9y5cicybrhhqsa95.png"
-  ],
-  "steelblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416197/amqyro3gix08x6shrfse.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416249/zunvoy8vibbzqefqfkg0.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416255/whzbzzogzo5d9u1s3oym.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416307/sxqy71iwrzngraaqy41z.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416257/zx2rocsa6yo0hlfr6g3f.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416172/ufxqq1uylrgqzklew8dx.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416227/sstrutfjlgnriihaeiqr.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416304/saebaj98hfibjsrxh6pe.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416282/n7j0vwkpwaw9gdh5yqh6.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416270/cujzcybg3letrklfedyq.png"
-  ],
-  "purple": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415976/c49c6b4ghcascmn4xfsm.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416276/zar1mfht0oqihxq7ciek.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416204/qknnwtey3qjb5madflre.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416330/khsiuv0wjbulqncixkxh.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416326/lvofqnvvvshtuacbat9c.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416217/bdwtuvpgbhbx7gjwlteb.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416280/t9udoglicwhgict1zcxf.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416218/kstch50r1aejy5lnqm8p.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416281/z2abttmsbynsnumwlqg3.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416257/nilon24mjwuwkewq0gae.png"
-  ],
-  "skyblue": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416235/kpslv6ns5dpnneniazhg.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416170/sfzqob28zvb9uw2sftum.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415967/cr1iwmrjopvh4oiz6tdg.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416202/r5vobz5we7aegrustg9y.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415983/fpryq4gkkdmkuoldsy7p.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415979/y9pwxvqyhqqiupsxoo78.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415960/i5ifavyrvgy1ay4u1isg.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416230/uydhjaphwoaowfm0sxzu.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416331/dqozvw2bjohcfo3zrwko.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416249/chdorgyrnfbpq49xgxew.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415998/i4wzvtqzfymknwyfuyc6.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416182/ztobiv6hgdafne2jw3s7.png"
-  ],
-  "aqua": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416340/h1kuqgcqpjzwu0ljgjzl.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416321/dzi2zp9sztzqtw9uee7r.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416174/ud2uehcqq1qyghq0utcp.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415964/ksisxgqdtz2vjyxxf0h5.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415963/op7g9sppryp1h2szkawc.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416330/odo3lr9n9qslrpelpf17.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416341/qq7aqw8a1tbjnzua5ofy.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416237/rlj8h5vqatrvid2htupx.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415962/lc02levu16k5xkcsdkqw.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416239/gnttl90pitpt5isdqvxb.png"
-  ],
-  "darkgreen": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416264/hgfibbhawru3agvmqhmp.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416251/neqrvs4qgeumrv4vfmwp.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416234/dgzqkw1d2n6ndcit4wnb.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416188/ug26ujte97hoqtgj8gxt.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416232/woljjv2lj53ioyvydv6b.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415972/apqgw44r8kjxf6wpevyl.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415968/mzxgjg1w67lfns5fcbsq.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416222/yoloxsbdp4fsergeernp.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416268/cjwpdaow3vxkyxv3n5pn.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415996/yczrjb9sqy1e1nhwcmq1.png"
-  ],
-  "violet": [
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416223/umysgecl2lxao9ujbupq.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416187/gn4k5mcwnhft4suls5r8.png",
-    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416275/aj6ismbfekdqh41mffaa.png"
-  ]
-}</t>
   </si>
   <si>
     <t>Chaqueta Yoga en licra</t>
@@ -2025,9 +1832,6 @@
   </si>
   <si>
     <t>Chaqueta en Algodón Perchado</t>
-  </si>
-  <si>
-    <t>L.XL</t>
   </si>
   <si>
     <t>{
@@ -2371,9 +2175,6 @@
 }</t>
   </si>
   <si>
-    <t>Enterizo 3 huecos</t>
-  </si>
-  <si>
     <t>blue,white,black</t>
   </si>
   <si>
@@ -2655,9 +2456,6 @@
     "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058817/xnmxv2e9memmagybowsd.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058816/s6zbit7x8tejpcfnv3s0.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058817/wqonc9kcviofhs7qiatn.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775058818/ht4eo6wpkw58c3zsjttb.png" ]}</t>
   </si>
   <si>
-    <t>{ "blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253382/k5shc79l7qjtrz6ci2u8.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662299/g4llyutemrjvlpsyhbjl.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662300/qtwerqw10yv6wxqpb1cl.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775267794/oq0hzp8xiepkigd8hytz.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662302/wghzvjuaajuwpbfddzvk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253384/fa3gtcxcbbujpmz1q32y.png"],"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662299/ys0v7pwpkcommwyjadtf.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662310/tbrnns244roeseqtkxrr.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253383/dxofsgljvhppxhvxcf9q.png"],"darkred":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253383/uqqd6kygifncoygwvzfk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253382/kiy5vdzzlhglrhntyfpf.png"], "royalblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662300/t7f9xsg5ij4gmjrmoyso.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662304/k5128obkwuopjaualtol.png"]}</t>
-  </si>
-  <si>
     <t>{
   "black": [
     "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774715391/agiednmodeb5yfpahlp1.png",
@@ -3210,6 +3008,226 @@
     "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775651819/wd6hvrxu5emoawuzy27y.png"
   ]
 }</t>
+  </si>
+  <si>
+    <t>{
+  "pink": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420046/o4phycvt82wjz8kplszr.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420265/twvchekif2zodyxanc1i.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713801/p2wxvvbmc7ugko9h06yo.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713802/umoe5klkejubiyq5x6qm.png"
+  ],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420039/zy4nsioggmxibakgkmnq.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420258/befqhobvwpandubpdwnx.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420208/nsi9nfrc9iwjh549x27f.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420041/oscbxkl0amqrovmxdl96.png"
+    ],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420271/emoayd31qpmmzq1e3cow.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420209/grarwuvkojfsxp3zkkea.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420219/iej9eryy6zmsqpxbtren.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420269/ssqsptxxtzk5242meapv.png"
+   ],
+  "green": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420212/dwppw1yttgi1glfoirjp.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420261/tsukkdewe1ssc9fx1xyf.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420213/nslqbwrpsalmznectkju.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420205/tjubdm4z489rrllcpjae.png"
+    ],
+  "darkblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420050/a3sah9k0vso0yczkejjp.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420217/qqxejrn7vafzp7mxinpd.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420203/tjmfayvfgtfwvotp3w7b.png" ],
+  "hotpink": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420202/mllthenng41x09edlbhz.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420045/a2ajlcckgz0jrgzkc5ym.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420259/rpf0na4o552r5leox8lp.png"  ],
+  "steelblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420215/ctwopprmeqldjrqo7ore.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773420277/vme2qfi6m8fkbpuuwwmw.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713803/wwstemtvnkfhxfdsqyja.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713802/lnhhqbsbq7hh058lp3s7.png"
+  ]}</t>
+  </si>
+  <si>
+    <t>{
+  "pink": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072753/dsppjvpwowbghyyabeog.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072754/iufnbxgh8v2t6nun4m8f.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072791/lycg5baqgojxovlk3klq.png"
+  ],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072764/q9ui9mat04sqcn7jpqb8.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072753/vaefzvoqosvza2tjc04h.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072751/tktrkjoftskg81kjytab.png"
+    ],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072762/oxepi3ridavl6iaquioe.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072768/jibcdv8zdbbnl2shknx5.png",  "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072784/lkxruusxffwbja8pvoem.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072794/htikpbl3pq2mpqp2ps8r.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072753/egdi0tylliek1qyjso6x.png"
+   ],
+  "green": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072758/tfir7j2qcftiffz8aca6.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072757/schvcegqk9teituzut2v.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072772/fuhllgv2gcygjv5uvhqx.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072786/iulimynpkmgyp1lrfyca.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072787/fhvdbb22uf43y6a8y3pz.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072763/xjzgglbt4ryzsr1dvjul.png"
+    ],
+  "darkblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072771/ocuhg6y7bx3q4k6qswwm.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072761/to6r3iw5czbnugwicbyo.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072755/njj3ykdg4wphlwueohpp.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072772/smojgyyxywm1ppopmhac.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072766/ehfpqr0onlnnfcmxkw6g.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072765/aijvgan44bsdlarde9hu.png"],
+  "hotpink": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072776/xy0oq8u2z354b9irwdi0.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072760/f7qv7ihynasmahakerzr.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072759/khvijabocbvnua4rq4vt.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072778/mey8d1cqjigzohe2kfsh.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072791/pglujdgbvmqn12el2igs.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072752/lud7tphmwdzz98gq2bkm.png"  ],
+  "steelblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072778/rt8jsbd8g77dtmflde6n.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072783/qzzslyqihjzfteprnqu3.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072756/nrlasih250wtk3djzpne.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1772072781/ecdvpj1gcs5bf219hskg.png"
+  ]}</t>
+  </si>
+  <si>
+    <t>{
+  "pink": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416290/qrlowbtwfkpfypavclt5.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416053/k746fugxvqwjknpiychz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416262/wqdfvzcho2lfxta4gzgz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416311/ooa4txwpixsa1zktiz0o.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416250/ets5y8x1rkziuisz27vd.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416286/bn9euxkqhrbqlmvuhxiz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416207/bmecxkohc2lcciefvprm.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416302/fc0pvuenvqudhe0ry818.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416195/kqzwt4sp5q0ge1hh8dwq.png"
+  ],
+  "blue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416294/pmshoq3tjgafq6gpcbt9.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416273/uogfsfsucmmsnyepdtbb.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416220/jdzz1cc3iaizq4j4dz6e.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416183/filmlgbtdgt2pd2pjeuo.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416323/qmthfapue8mwtsxurtfz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416244/vxyttjxduexjvje1lvm6.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416215/snrk8fldawf0oirrvquv.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416178/pr4qhmhhxtvt0d5apipa.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415980/gzezgzr4ue2yp3mu5rzo.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416196/f9jdzglnonjv9mrqmrea.png"
+  ],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415970/j0emdwlkpwvkwyofrxkv.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416208/jksbv56emig4qz94gmu9.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415974/zlvlfegmwgwtj3uegmf6.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416294/gom3hdiys0lpegiucrfa.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416262/hqptcmqk7le05zjivb2k.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416312/tbaamx57e76vf6gpb7wz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416316/yvchju9wkaf9elfxm2w6.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416263/xdmzoozc7dhxq6cuze6i.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416320/iq8yndysogkwqyeie3t1.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415991/t796xjnfo98lb7bhmvsq.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416310/ohb69dmxvobxucufp8fz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416289/hycllrw7ygufhch0nysq.png"
+  ],
+  "green": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416166/qrqgdfj7kqlb9zfng6og.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415990/j3al7u3gj7mkaku0qoby.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415980/cnnqftkwrshlexyjlapl.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415959/kjxny6jnzipqvk91ok2x.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415995/na8186pgdaqwniyxhose.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416176/s1w9mmdlhvuqb2avrrad.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415984/dpccybijitpf8ji3iteu.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416285/ybuu7gx8wzf3jejflzts.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416187/vioijghseh9sdqf2nkal.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416300/divgdwrvstqluscll2lf.png"
+  ],
+  "darkblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416299/fpqonbmnz6qfdppdzmsl.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416295/cwxjgbndrpebrw4dya7c.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416272/yutx8qm1vkjeggh99ew7.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416177/gsen39sqfogt42jmlpez.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415973/voeon9pukrdqtvq128kv.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416211/ubqgbda3rjout3urkw09.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416168/se1krtmrlk6epe6mmqzz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416242/wtlrtruu93kuzt61p55z.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416243/fcuvs7v55a66f46l0jed.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416310/bjypkov8tqc4gvms7tod.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415965/cvx3oyygwzfxfgj3mgof.png"
+  ],
+  "hotpink": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415987/iuyjozzwro18snorgkaz.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416003/vou1uotpawlgvdow6blj.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416228/grpnayzcsu7pwysdpm9l.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416336/so117psdpsxbfxn86aa4.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416212/clo6omrpdsqacmfbyx2e.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416003/nal0y1aousnydel9c9bh.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416167/wh3yinojxhalhz4qe3rg.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416180/yariiiyggalcawpthysm.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416317/eonvxsrpzrhn2vlcjatj.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416203/lv6d9y5cicybrhhqsa95.png"
+  ],
+  "steelblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416197/amqyro3gix08x6shrfse.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416249/zunvoy8vibbzqefqfkg0.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416255/whzbzzogzo5d9u1s3oym.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416307/sxqy71iwrzngraaqy41z.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416257/zx2rocsa6yo0hlfr6g3f.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416172/ufxqq1uylrgqzklew8dx.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416227/sstrutfjlgnriihaeiqr.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416304/saebaj98hfibjsrxh6pe.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416282/n7j0vwkpwaw9gdh5yqh6.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416270/cujzcybg3letrklfedyq.png"
+  ],
+  "purple": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415976/c49c6b4ghcascmn4xfsm.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416276/zar1mfht0oqihxq7ciek.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416204/qknnwtey3qjb5madflre.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416330/khsiuv0wjbulqncixkxh.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416326/lvofqnvvvshtuacbat9c.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416217/bdwtuvpgbhbx7gjwlteb.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416280/t9udoglicwhgict1zcxf.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416218/kstch50r1aejy5lnqm8p.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416281/z2abttmsbynsnumwlqg3.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416257/nilon24mjwuwkewq0gae.png"
+  ],
+  "skyblue": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416235/kpslv6ns5dpnneniazhg.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416170/sfzqob28zvb9uw2sftum.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415967/cr1iwmrjopvh4oiz6tdg.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416202/r5vobz5we7aegrustg9y.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415983/fpryq4gkkdmkuoldsy7p.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415979/y9pwxvqyhqqiupsxoo78.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415960/i5ifavyrvgy1ay4u1isg.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416230/uydhjaphwoaowfm0sxzu.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416331/dqozvw2bjohcfo3zrwko.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416249/chdorgyrnfbpq49xgxew.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415998/i4wzvtqzfymknwyfuyc6.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416182/ztobiv6hgdafne2jw3s7.png"
+  ],
+  "aqua": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416340/h1kuqgcqpjzwu0ljgjzl.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416321/dzi2zp9sztzqtw9uee7r.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416174/ud2uehcqq1qyghq0utcp.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415964/ksisxgqdtz2vjyxxf0h5.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415963/op7g9sppryp1h2szkawc.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416330/odo3lr9n9qslrpelpf17.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416341/qq7aqw8a1tbjnzua5ofy.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416237/rlj8h5vqatrvid2htupx.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415962/lc02levu16k5xkcsdkqw.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416239/gnttl90pitpt5isdqvxb.png"
+  ],
+  "darkgreen": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416264/hgfibbhawru3agvmqhmp.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416251/neqrvs4qgeumrv4vfmwp.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416234/dgzqkw1d2n6ndcit4wnb.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416188/ug26ujte97hoqtgj8gxt.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416232/woljjv2lj53ioyvydv6b.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415972/apqgw44r8kjxf6wpevyl.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415968/mzxgjg1w67lfns5fcbsq.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416222/yoloxsbdp4fsergeernp.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416268/cjwpdaow3vxkyxv3n5pn.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773415996/yczrjb9sqy1e1nhwcmq1.png"
+  ],
+  "violet": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416223/umysgecl2lxao9ujbupq.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416187/gn4k5mcwnhft4suls5r8.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773416275/aj6ismbfekdqh41mffaa.png"
+  ]
+}</t>
+  </si>
+  <si>
+    <t>{ "blue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253382/k5shc79l7qjtrz6ci2u8.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662299/g4llyutemrjvlpsyhbjl.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662300/qtwerqw10yv6wxqpb1cl.png"],"red":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775267794/oq0hzp8xiepkigd8hytz.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662302/wghzvjuaajuwpbfddzvk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253384/fa3gtcxcbbujpmz1q32y.png"],"black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775714831/nhh5gtcr98xedfimwedl.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662310/tbrnns244roeseqtkxrr.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253383/dxofsgljvhppxhvxcf9q.png"],"darkred":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253383/uqqd6kygifncoygwvzfk.png","https://res.cloudinary.com/dtwqvxhnm/image/upload/v1773253382/kiy5vdzzlhglrhntyfpf.png"], "royalblue":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662300/t7f9xsg5ij4gmjrmoyso.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1774662304/k5128obkwuopjaualtol.png"]}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pantaloneta Running </t>
+  </si>
+  <si>
+    <t>olive,red,gray,crimson,purple,black</t>
+  </si>
+  <si>
+    <t>{
+  "olive": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713346/tirpl3vsebbxrpsfldwa.png",
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713346/lw9j7utvommec2ljjdiz.png"
+  ],
+  "red": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713349/zpibbakrvtjje3uwbvzm.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713347/msywbixpzz0lwwozubzc.png"  ],
+  "gray": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713349/qb9trx4cyydbujc20cyz.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713348/wholmpws1svmvxqluujx.png"  ],
+  "crimson": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713351/byvtbwdxluxnxvkvux3v.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713349/yss9zulo0nkd0he9rkan.png"  ],
+  "purple": [
+    "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713350/uns1jry9u4vcyoyupwtd.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713347/xfvipr4dadf6rc2qpct4.png"], "black":["https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713350/xnyrgtj0p8li9nkwj020.png", "https://res.cloudinary.com/dtwqvxhnm/image/upload/v1775713350/g8mxtmqu5p9mwegpqbnz.png"   ]
+  }</t>
+  </si>
+  <si>
+    <t>Rompevientos Malla Interna</t>
+  </si>
+  <si>
+    <t>Enterizo Tentación</t>
   </si>
 </sst>
 </file>
@@ -3233,7 +3251,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3288,6 +3306,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -3316,7 +3340,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -3397,6 +3421,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3705,7 +3735,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D9C4F76-C123-4A10-B08E-8C496E2AA870}">
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="57.54296875" style="2" customWidth="1"/>
@@ -3726,7 +3756,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
@@ -3764,10 +3794,10 @@
         <v>16</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>11</v>
@@ -3785,10 +3815,10 @@
         <v>17</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="K2" s="6" t="b">
         <v>0</v>
@@ -3799,13 +3829,13 @@
     </row>
     <row r="3" spans="1:12" s="3" customFormat="1" ht="99.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>11</v>
@@ -3821,10 +3851,10 @@
         <v>14</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="K3" s="6" t="b">
         <v>0</v>
@@ -3835,13 +3865,13 @@
     </row>
     <row r="4" spans="1:12" s="3" customFormat="1" ht="89.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>11</v>
@@ -3859,10 +3889,10 @@
         <v>17</v>
       </c>
       <c r="I4" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>69</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>70</v>
       </c>
       <c r="K4" s="6" t="b">
         <v>0</v>
@@ -3876,10 +3906,10 @@
         <v>19</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>20</v>
@@ -3897,10 +3927,10 @@
         <v>17</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="K5" s="6" t="b">
         <v>0</v>
@@ -3915,7 +3945,7 @@
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>11</v>
@@ -3931,10 +3961,10 @@
         <v>14</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="K6" s="6" t="b">
         <v>0</v>
@@ -3945,11 +3975,11 @@
     </row>
     <row r="7" spans="1:12" ht="77.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>11</v>
@@ -3965,10 +3995,10 @@
         <v>12</v>
       </c>
       <c r="I7" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="J7" s="11" t="s">
         <v>72</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>73</v>
       </c>
       <c r="K7" s="6" t="b">
         <v>0</v>
@@ -3983,7 +4013,7 @@
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>11</v>
@@ -4001,10 +4031,10 @@
         <v>13</v>
       </c>
       <c r="I8" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="J8" s="11" t="s">
         <v>74</v>
-      </c>
-      <c r="J8" s="11" t="s">
-        <v>75</v>
       </c>
       <c r="K8" s="6" t="b">
         <v>0</v>
@@ -4015,11 +4045,11 @@
     </row>
     <row r="9" spans="1:12" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>11</v>
@@ -4037,10 +4067,10 @@
         <v>13</v>
       </c>
       <c r="I9" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="J9" s="11" t="s">
         <v>74</v>
-      </c>
-      <c r="J9" s="11" t="s">
-        <v>75</v>
       </c>
       <c r="K9" s="6" t="b">
         <v>0</v>
@@ -4055,7 +4085,7 @@
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>11</v>
@@ -4071,10 +4101,10 @@
         <v>14</v>
       </c>
       <c r="I10" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="J10" s="12" t="s">
         <v>76</v>
-      </c>
-      <c r="J10" s="12" t="s">
-        <v>77</v>
       </c>
       <c r="K10" s="6" t="b">
         <v>0</v>
@@ -4085,11 +4115,11 @@
     </row>
     <row r="11" spans="1:12" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>11</v>
@@ -4105,10 +4135,10 @@
         <v>14</v>
       </c>
       <c r="I11" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="J11" s="12" t="s">
         <v>76</v>
-      </c>
-      <c r="J11" s="12" t="s">
-        <v>77</v>
       </c>
       <c r="K11" s="6" t="b">
         <v>0</v>
@@ -4119,11 +4149,11 @@
     </row>
     <row r="12" spans="1:12" ht="47" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>11</v>
@@ -4139,10 +4169,10 @@
         <v>14</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="K12" s="6" t="b">
         <v>0</v>
@@ -4153,11 +4183,11 @@
     </row>
     <row r="13" spans="1:12" ht="47" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>11</v>
@@ -4173,10 +4203,10 @@
         <v>14</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="K13" s="6" t="b">
         <v>0</v>
@@ -4187,11 +4217,11 @@
     </row>
     <row r="14" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>26</v>
@@ -4209,10 +4239,10 @@
         <v>25</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K14" s="6" t="b">
         <v>0</v>
@@ -4223,11 +4253,11 @@
     </row>
     <row r="15" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>26</v>
@@ -4245,10 +4275,10 @@
         <v>25</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K15" s="6" t="b">
         <v>0</v>
@@ -4259,11 +4289,11 @@
     </row>
     <row r="16" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>11</v>
@@ -4281,10 +4311,10 @@
         <v>25</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K16" s="6" t="b">
         <v>0</v>
@@ -4295,11 +4325,11 @@
     </row>
     <row r="17" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>11</v>
@@ -4317,10 +4347,10 @@
         <v>25</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K17" s="6" t="b">
         <v>0</v>
@@ -4335,7 +4365,7 @@
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>29</v>
@@ -4351,10 +4381,10 @@
         <v>27</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K18" s="6" t="b">
         <v>0</v>
@@ -4365,7 +4395,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="6" t="s">
@@ -4385,10 +4415,10 @@
         <v>27</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K19" s="6" t="b">
         <v>0</v>
@@ -4399,11 +4429,11 @@
     </row>
     <row r="20" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>11</v>
@@ -4419,10 +4449,10 @@
         <v>14</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K20" s="6" t="b">
         <v>0</v>
@@ -4437,7 +4467,7 @@
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>11</v>
@@ -4453,10 +4483,10 @@
         <v>14</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J21" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K21" s="6" t="b">
         <v>0</v>
@@ -4471,7 +4501,7 @@
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>11</v>
@@ -4487,10 +4517,10 @@
         <v>31</v>
       </c>
       <c r="I22" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="J22" s="12" t="s">
         <v>128</v>
-      </c>
-      <c r="J22" s="12" t="s">
-        <v>129</v>
       </c>
       <c r="K22" s="6" t="b">
         <v>0</v>
@@ -4505,7 +4535,7 @@
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>11</v>
@@ -4521,10 +4551,10 @@
         <v>14</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J23" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K23" s="6" t="b">
         <v>0</v>
@@ -4539,7 +4569,7 @@
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>11</v>
@@ -4555,10 +4585,10 @@
         <v>14</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J24" s="12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K24" s="6" t="b">
         <v>0</v>
@@ -4573,7 +4603,7 @@
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>11</v>
@@ -4589,10 +4619,10 @@
         <v>14</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="K25" s="6" t="b">
         <v>0</v>
@@ -4603,7 +4633,7 @@
     </row>
     <row r="26" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6" t="s">
@@ -4623,10 +4653,10 @@
         <v>14</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="K26" s="6" t="b">
         <v>0</v>
@@ -4641,7 +4671,7 @@
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>11</v>
@@ -4657,10 +4687,10 @@
         <v>14</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="K27" s="6" t="b">
         <v>0</v>
@@ -4675,7 +4705,7 @@
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>11</v>
@@ -4691,10 +4721,10 @@
         <v>14</v>
       </c>
       <c r="I28" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="J28" s="12" t="s">
         <v>85</v>
-      </c>
-      <c r="J28" s="12" t="s">
-        <v>86</v>
       </c>
       <c r="K28" s="6" t="b">
         <v>0</v>
@@ -4705,7 +4735,7 @@
     </row>
     <row r="29" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="6" t="s">
@@ -4725,10 +4755,10 @@
         <v>40</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J29" s="12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K29" s="6" t="b">
         <v>0</v>
@@ -4739,7 +4769,7 @@
     </row>
     <row r="30" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="6" t="s">
@@ -4759,10 +4789,10 @@
         <v>40</v>
       </c>
       <c r="I30" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="J30" s="12" t="s">
         <v>88</v>
-      </c>
-      <c r="J30" s="12" t="s">
-        <v>89</v>
       </c>
       <c r="K30" s="6" t="b">
         <v>0</v>
@@ -4795,10 +4825,10 @@
         <v>43</v>
       </c>
       <c r="I31" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="J31" s="12" t="s">
         <v>90</v>
-      </c>
-      <c r="J31" s="12" t="s">
-        <v>91</v>
       </c>
       <c r="K31" s="6" t="b">
         <v>0</v>
@@ -4831,10 +4861,10 @@
         <v>44</v>
       </c>
       <c r="I32" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="J32" s="12" t="s">
         <v>92</v>
-      </c>
-      <c r="J32" s="12" t="s">
-        <v>93</v>
       </c>
       <c r="K32" s="6" t="b">
         <v>0</v>
@@ -4865,10 +4895,10 @@
         <v>14</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="K33" s="6" t="b">
         <v>0</v>
@@ -4899,10 +4929,10 @@
         <v>14</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="K34" s="6" t="b">
         <v>0</v>
@@ -4913,7 +4943,7 @@
     </row>
     <row r="35" spans="1:12" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="6" t="s">
@@ -4926,7 +4956,7 @@
         <v>17000</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G35" s="6">
         <v>34000</v>
@@ -4935,10 +4965,10 @@
         <v>40</v>
       </c>
       <c r="I35" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J35" s="8" t="s">
         <v>95</v>
-      </c>
-      <c r="J35" s="8" t="s">
-        <v>96</v>
       </c>
       <c r="K35" s="6" t="b">
         <v>0</v>
@@ -4949,7 +4979,7 @@
     </row>
     <row r="36" spans="1:12" ht="126.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="6" t="s">
@@ -4962,7 +4992,7 @@
         <v>17000</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G36" s="6">
         <v>34000</v>
@@ -4971,10 +5001,10 @@
         <v>40</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J36" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K36" s="6" t="b">
         <v>0</v>
@@ -4985,7 +5015,7 @@
     </row>
     <row r="37" spans="1:12" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6" t="s">
@@ -4998,7 +5028,7 @@
         <v>17000</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G37" s="6">
         <v>34000</v>
@@ -5007,10 +5037,10 @@
         <v>40</v>
       </c>
       <c r="I37" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J37" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K37" s="6" t="b">
         <v>0</v>
@@ -5021,7 +5051,7 @@
     </row>
     <row r="38" spans="1:12" ht="91" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="6" t="s">
@@ -5034,7 +5064,7 @@
         <v>17000</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G38" s="6">
         <v>34000</v>
@@ -5043,10 +5073,10 @@
         <v>40</v>
       </c>
       <c r="I38" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="J38" s="8" t="s">
         <v>99</v>
-      </c>
-      <c r="J38" s="8" t="s">
-        <v>100</v>
       </c>
       <c r="K38" s="6" t="b">
         <v>0</v>
@@ -5057,7 +5087,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="6" t="s">
@@ -5077,10 +5107,10 @@
         <v>51</v>
       </c>
       <c r="I39" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="J39" s="12" t="s">
         <v>101</v>
-      </c>
-      <c r="J39" s="12" t="s">
-        <v>102</v>
       </c>
       <c r="K39" s="6" t="b">
         <v>0</v>
@@ -5111,10 +5141,10 @@
         <v>51</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J40" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K40" s="6" t="b">
         <v>0</v>
@@ -5125,7 +5155,7 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A41" s="6" t="s">
-        <v>52</v>
+        <v>369</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="6" t="s">
@@ -5145,10 +5175,10 @@
         <v>14</v>
       </c>
       <c r="I41" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="J41" s="14" t="s">
         <v>104</v>
-      </c>
-      <c r="J41" s="14" t="s">
-        <v>105</v>
       </c>
       <c r="K41" s="6" t="b">
         <v>0</v>
@@ -5159,7 +5189,7 @@
     </row>
     <row r="42" spans="1:12" ht="98.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="6" t="s">
@@ -5179,10 +5209,10 @@
         <v>44</v>
       </c>
       <c r="I42" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J42" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K42" s="6" t="b">
         <v>0</v>
@@ -5193,7 +5223,7 @@
     </row>
     <row r="43" spans="1:12" ht="95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="6" t="s">
@@ -5213,10 +5243,10 @@
         <v>44</v>
       </c>
       <c r="I43" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J43" s="15" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="K43" s="6" t="b">
         <v>0</v>
@@ -5227,7 +5257,7 @@
     </row>
     <row r="44" spans="1:12" ht="158" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="6" t="s">
@@ -5247,10 +5277,10 @@
         <v>14</v>
       </c>
       <c r="I44" s="7" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="J44" s="8" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="K44" s="6" t="b">
         <v>0</v>
@@ -5274,19 +5304,19 @@
         <v>10000</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G45" s="6">
         <v>19000</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I45" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="J45" s="8" t="s">
         <v>108</v>
-      </c>
-      <c r="J45" s="8" t="s">
-        <v>109</v>
       </c>
       <c r="K45" s="6" t="b">
         <v>0</v>
@@ -5297,7 +5327,7 @@
     </row>
     <row r="46" spans="1:12" ht="82" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="6" t="s">
@@ -5314,13 +5344,13 @@
         <v>20000</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I46" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="J46" s="8" t="s">
         <v>110</v>
-      </c>
-      <c r="J46" s="8" t="s">
-        <v>111</v>
       </c>
       <c r="K46" s="6" t="b">
         <v>0</v>
@@ -5331,7 +5361,7 @@
     </row>
     <row r="47" spans="1:12" ht="302.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="6" t="s">
@@ -5351,10 +5381,10 @@
         <v>13</v>
       </c>
       <c r="I47" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J47" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K47" s="6" t="b">
         <v>0</v>
@@ -5365,7 +5395,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="6" t="s">
@@ -5382,13 +5412,13 @@
         <v>30000</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I48" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="J48" s="14" t="s">
         <v>113</v>
-      </c>
-      <c r="J48" s="14" t="s">
-        <v>114</v>
       </c>
       <c r="K48" s="6" t="b">
         <v>0</v>
@@ -5399,7 +5429,7 @@
     </row>
     <row r="49" spans="1:12" ht="261.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="6" t="s">
@@ -5419,10 +5449,10 @@
         <v>12</v>
       </c>
       <c r="I49" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J49" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K49" s="6" t="b">
         <v>0</v>
@@ -5433,11 +5463,11 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A50" s="6" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>11</v>
@@ -5453,10 +5483,10 @@
         <v>12</v>
       </c>
       <c r="I50" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="J50" s="14" t="s">
         <v>116</v>
-      </c>
-      <c r="J50" s="14" t="s">
-        <v>117</v>
       </c>
       <c r="K50" s="6" t="b">
         <v>0</v>
@@ -5467,7 +5497,7 @@
     </row>
     <row r="51" spans="1:12" ht="406" x14ac:dyDescent="0.35">
       <c r="A51" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="6" t="s">
@@ -5487,10 +5517,10 @@
         <v>12</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="J51" s="8" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="K51" s="6" t="b">
         <v>0</v>
@@ -5501,7 +5531,7 @@
     </row>
     <row r="52" spans="1:12" ht="121.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="6" t="s">
@@ -5521,10 +5551,10 @@
         <v>14</v>
       </c>
       <c r="I52" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J52" s="15" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="K52" s="6" t="b">
         <v>0</v>
@@ -5535,11 +5565,11 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A53" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>11</v>
@@ -5555,10 +5585,10 @@
         <v>14</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J53" s="12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K53" s="6" t="b">
         <v>0</v>
@@ -5569,11 +5599,11 @@
     </row>
     <row r="54" spans="1:12" ht="141.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D54" s="6" t="s">
         <v>11</v>
@@ -5589,10 +5619,10 @@
         <v>14</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K54" s="6" t="b">
         <v>0</v>
@@ -5603,11 +5633,11 @@
     </row>
     <row r="55" spans="1:12" ht="276.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>11</v>
@@ -5623,10 +5653,10 @@
         <v>14</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K55" s="6" t="b">
         <v>0</v>
@@ -5637,11 +5667,11 @@
     </row>
     <row r="56" spans="1:12" ht="42.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D56" s="6" t="s">
         <v>11</v>
@@ -5657,10 +5687,10 @@
         <v>31</v>
       </c>
       <c r="I56" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="J56" s="6" t="s">
         <v>122</v>
-      </c>
-      <c r="J56" s="6" t="s">
-        <v>123</v>
       </c>
       <c r="K56" s="6" t="b">
         <v>0</v>
@@ -5671,11 +5701,11 @@
     </row>
     <row r="57" spans="1:12" ht="377" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>11</v>
@@ -5684,7 +5714,7 @@
         <v>22000</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G57" s="6">
         <v>27000</v>
@@ -5693,10 +5723,10 @@
         <v>17</v>
       </c>
       <c r="I57" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="J57" s="15" t="s">
         <v>166</v>
-      </c>
-      <c r="J57" s="15" t="s">
-        <v>167</v>
       </c>
       <c r="K57" s="6" t="b">
         <v>0</v>
@@ -5707,11 +5737,11 @@
     </row>
     <row r="58" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A58" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B58" s="16"/>
       <c r="C58" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D58" s="16" t="s">
         <v>26</v>
@@ -5727,10 +5757,10 @@
         <v>14</v>
       </c>
       <c r="I58" s="17" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J58" s="18" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="K58" s="19" t="b">
         <v>0</v>
@@ -5741,11 +5771,11 @@
     </row>
     <row r="59" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A59" s="16" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B59" s="16"/>
       <c r="C59" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D59" s="16" t="s">
         <v>20</v>
@@ -5761,10 +5791,10 @@
         <v>14</v>
       </c>
       <c r="I59" s="17" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J59" s="18" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K59" s="19" t="b">
         <v>0</v>
@@ -5775,11 +5805,11 @@
     </row>
     <row r="60" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A60" s="16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B60" s="16"/>
       <c r="C60" s="16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D60" s="16" t="s">
         <v>20</v>
@@ -5795,10 +5825,10 @@
         <v>14</v>
       </c>
       <c r="I60" s="17" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J60" s="18" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="K60" s="19" t="b">
         <v>0</v>
@@ -5809,11 +5839,11 @@
     </row>
     <row r="61" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A61" s="16" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B61" s="16"/>
       <c r="C61" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D61" s="16" t="s">
         <v>20</v>
@@ -5829,10 +5859,10 @@
         <v>14</v>
       </c>
       <c r="I61" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J61" s="18" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K61" s="19" t="b">
         <v>0</v>
@@ -5843,11 +5873,11 @@
     </row>
     <row r="62" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A62" s="16" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D62" s="16" t="s">
         <v>20</v>
@@ -5863,10 +5893,10 @@
         <v>14</v>
       </c>
       <c r="I62" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="J62" s="18" t="s">
         <v>183</v>
-      </c>
-      <c r="J62" s="18" t="s">
-        <v>184</v>
       </c>
       <c r="K62" s="19" t="b">
         <v>0</v>
@@ -5877,11 +5907,11 @@
     </row>
     <row r="63" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A63" s="16" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B63" s="16"/>
       <c r="C63" s="16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D63" s="16" t="s">
         <v>20</v>
@@ -5897,10 +5927,10 @@
         <v>14</v>
       </c>
       <c r="I63" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="J63" s="18" t="s">
         <v>189</v>
-      </c>
-      <c r="J63" s="18" t="s">
-        <v>190</v>
       </c>
       <c r="K63" s="19" t="b">
         <v>0</v>
@@ -5911,11 +5941,11 @@
     </row>
     <row r="64" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A64" s="16" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B64" s="16"/>
       <c r="C64" s="16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D64" s="16" t="s">
         <v>20</v>
@@ -5931,10 +5961,10 @@
         <v>14</v>
       </c>
       <c r="I64" s="17" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J64" s="18" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K64" s="19" t="b">
         <v>0</v>
@@ -5945,11 +5975,11 @@
     </row>
     <row r="65" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A65" s="16" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B65" s="16"/>
       <c r="C65" s="16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D65" s="16" t="s">
         <v>20</v>
@@ -5965,10 +5995,10 @@
         <v>14</v>
       </c>
       <c r="I65" s="17" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J65" s="18" t="s">
-        <v>205</v>
+        <v>364</v>
       </c>
       <c r="K65" s="19" t="b">
         <v>0</v>
@@ -5979,11 +6009,11 @@
     </row>
     <row r="66" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A66" s="16" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B66" s="16"/>
       <c r="C66" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D66" s="16" t="s">
         <v>20</v>
@@ -5999,10 +6029,10 @@
         <v>14</v>
       </c>
       <c r="I66" s="17" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="J66" s="18" t="s">
-        <v>204</v>
+        <v>363</v>
       </c>
       <c r="K66" s="19" t="b">
         <v>0</v>
@@ -6013,11 +6043,11 @@
     </row>
     <row r="67" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A67" s="16" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B67" s="16"/>
       <c r="C67" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D67" s="16" t="s">
         <v>20</v>
@@ -6033,10 +6063,10 @@
         <v>14</v>
       </c>
       <c r="I67" s="17" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="J67" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K67" s="19" t="b">
         <v>0</v>
@@ -6047,11 +6077,11 @@
     </row>
     <row r="68" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A68" s="16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B68" s="16"/>
       <c r="C68" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D68" s="16" t="s">
         <v>20</v>
@@ -6067,10 +6097,10 @@
         <v>14</v>
       </c>
       <c r="I68" s="17" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="J68" s="18" t="s">
-        <v>201</v>
+        <v>362</v>
       </c>
       <c r="K68" s="19" t="b">
         <v>0</v>
@@ -6081,11 +6111,11 @@
     </row>
     <row r="69" spans="1:12" ht="406" x14ac:dyDescent="0.35">
       <c r="A69" s="16" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B69" s="16"/>
       <c r="C69" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D69" s="16" t="s">
         <v>20</v>
@@ -6101,10 +6131,10 @@
         <v>14</v>
       </c>
       <c r="I69" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J69" s="18" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K69" s="19" t="b">
         <v>0</v>
@@ -6115,11 +6145,11 @@
     </row>
     <row r="70" spans="1:12" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A70" s="16" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B70" s="16"/>
       <c r="C70" s="16" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D70" s="16" t="s">
         <v>20</v>
@@ -6135,10 +6165,10 @@
         <v>14</v>
       </c>
       <c r="I70" s="16" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="J70" s="17" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="K70" s="19" t="b">
         <v>0</v>
@@ -6149,11 +6179,11 @@
     </row>
     <row r="71" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A71" s="16" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B71" s="16"/>
       <c r="C71" s="16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D71" s="16" t="s">
         <v>20</v>
@@ -6169,10 +6199,10 @@
         <v>14</v>
       </c>
       <c r="I71" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J71" s="18" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="K71" s="19" t="b">
         <v>0</v>
@@ -6183,11 +6213,11 @@
     </row>
     <row r="72" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A72" s="16" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B72" s="16"/>
       <c r="C72" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D72" s="16" t="s">
         <v>20</v>
@@ -6203,10 +6233,10 @@
         <v>14</v>
       </c>
       <c r="I72" s="17" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J72" s="18" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="K72" s="19" t="b">
         <v>0</v>
@@ -6217,11 +6247,11 @@
     </row>
     <row r="73" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A73" s="16" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B73" s="16"/>
       <c r="C73" s="16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D73" s="16" t="s">
         <v>20</v>
@@ -6237,10 +6267,10 @@
         <v>14</v>
       </c>
       <c r="I73" s="17" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J73" s="18" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="K73" s="19" t="b">
         <v>0</v>
@@ -6251,13 +6281,13 @@
     </row>
     <row r="74" spans="1:12" ht="319" x14ac:dyDescent="0.35">
       <c r="A74" s="16" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="B74" s="17" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="C74" s="16" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D74" s="16" t="s">
         <v>11</v>
@@ -6270,13 +6300,13 @@
         <v>34000</v>
       </c>
       <c r="H74" s="16" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="I74" s="16" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J74" s="18" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="K74" s="19" t="b">
         <v>0</v>
@@ -6287,11 +6317,11 @@
     </row>
     <row r="75" spans="1:12" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A75" s="16" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B75" s="16"/>
       <c r="C75" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D75" s="16" t="s">
         <v>20</v>
@@ -6307,10 +6337,10 @@
         <v>14</v>
       </c>
       <c r="I75" s="16" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="J75" s="18" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="K75" s="19" t="b">
         <v>0</v>
@@ -6321,11 +6351,11 @@
     </row>
     <row r="76" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A76" s="16" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B76" s="16"/>
       <c r="C76" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D76" s="16" t="s">
         <v>20</v>
@@ -6341,10 +6371,10 @@
         <v>14</v>
       </c>
       <c r="I76" s="17" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="J76" s="17" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="K76" s="19" t="b">
         <v>0</v>
@@ -6355,11 +6385,11 @@
     </row>
     <row r="77" spans="1:12" ht="87" x14ac:dyDescent="0.35">
       <c r="A77" s="16" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B77" s="16"/>
       <c r="C77" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D77" s="16" t="s">
         <v>20</v>
@@ -6375,10 +6405,10 @@
         <v>14</v>
       </c>
       <c r="I77" s="16" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="J77" s="18" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="K77" s="19" t="b">
         <v>0</v>
@@ -6389,13 +6419,13 @@
     </row>
     <row r="78" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A78" s="16" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B78" s="16" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C78" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D78" s="16" t="s">
         <v>20</v>
@@ -6411,10 +6441,10 @@
         <v>14</v>
       </c>
       <c r="I78" s="17" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="J78" s="18" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="K78" s="19" t="b">
         <v>0</v>
@@ -6425,13 +6455,13 @@
     </row>
     <row r="79" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A79" s="16" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="B79" s="16" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C79" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D79" s="16" t="s">
         <v>20</v>
@@ -6447,10 +6477,10 @@
         <v>14</v>
       </c>
       <c r="I79" s="17" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="J79" s="18" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="K79" s="19" t="b">
         <v>0</v>
@@ -6461,11 +6491,11 @@
     </row>
     <row r="80" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A80" s="16" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B80" s="16"/>
       <c r="C80" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D80" s="16" t="s">
         <v>20</v>
@@ -6481,10 +6511,10 @@
         <v>14</v>
       </c>
       <c r="I80" s="16" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="J80" s="17" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="K80" s="19" t="b">
         <v>0</v>
@@ -6495,11 +6525,11 @@
     </row>
     <row r="81" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A81" s="16" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="B81" s="16"/>
       <c r="C81" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D81" s="16" t="s">
         <v>20</v>
@@ -6515,10 +6545,10 @@
         <v>14</v>
       </c>
       <c r="I81" s="16" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="J81" s="17" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="K81" s="19" t="b">
         <v>0</v>
@@ -6529,11 +6559,11 @@
     </row>
     <row r="82" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A82" s="16" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="B82" s="16"/>
       <c r="C82" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D82" s="16" t="s">
         <v>20</v>
@@ -6549,10 +6579,10 @@
         <v>14</v>
       </c>
       <c r="I82" s="17" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="J82" s="18" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="K82" s="19" t="b">
         <v>0</v>
@@ -6563,11 +6593,11 @@
     </row>
     <row r="83" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A83" s="16" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B83" s="16"/>
       <c r="C83" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D83" s="16" t="s">
         <v>20</v>
@@ -6583,10 +6613,10 @@
         <v>14</v>
       </c>
       <c r="I83" s="17" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="J83" s="21" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="K83" s="19" t="b">
         <v>0</v>
@@ -6597,11 +6627,11 @@
     </row>
     <row r="84" spans="1:12" ht="261" x14ac:dyDescent="0.35">
       <c r="A84" s="16" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="B84" s="16"/>
       <c r="C84" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D84" s="16" t="s">
         <v>20</v>
@@ -6617,10 +6647,10 @@
         <v>14</v>
       </c>
       <c r="I84" s="16" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="J84" s="21" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="K84" s="19" t="b">
         <v>0</v>
@@ -6631,11 +6661,11 @@
     </row>
     <row r="85" spans="1:12" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A85" s="16" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B85" s="16"/>
       <c r="C85" s="16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D85" s="16" t="s">
         <v>20</v>
@@ -6644,7 +6674,7 @@
         <v>25000</v>
       </c>
       <c r="F85" s="17" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="G85" s="16">
         <v>36000</v>
@@ -6653,10 +6683,10 @@
         <v>13</v>
       </c>
       <c r="I85" s="16" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="J85" s="21" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="K85" s="19" t="b">
         <v>0</v>
@@ -6667,11 +6697,11 @@
     </row>
     <row r="86" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A86" s="16" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B86" s="16"/>
       <c r="C86" s="16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D86" s="16" t="s">
         <v>20</v>
@@ -6687,10 +6717,10 @@
         <v>14</v>
       </c>
       <c r="I86" s="17" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="J86" s="21" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="K86" s="19" t="b">
         <v>0</v>
@@ -6701,11 +6731,11 @@
     </row>
     <row r="87" spans="1:12" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A87" s="6" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D87" s="6" t="s">
         <v>11</v>
@@ -6721,10 +6751,10 @@
         <v>12</v>
       </c>
       <c r="I87" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="J87" s="11" t="s">
         <v>72</v>
-      </c>
-      <c r="J87" s="11" t="s">
-        <v>73</v>
       </c>
       <c r="K87" s="6" t="b">
         <v>0</v>
@@ -6735,7 +6765,7 @@
     </row>
     <row r="88" spans="1:12" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A88" s="6" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="B88" s="6"/>
       <c r="C88" s="6" t="s">
@@ -6752,13 +6782,13 @@
         <v>27000</v>
       </c>
       <c r="H88" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="I88" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="J88" s="22" t="s">
         <v>265</v>
-      </c>
-      <c r="I88" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="J88" s="22" t="s">
-        <v>269</v>
       </c>
       <c r="K88" s="6" t="b">
         <v>0</v>
@@ -6769,7 +6799,7 @@
     </row>
     <row r="89" spans="1:12" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A89" s="6" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B89" s="6"/>
       <c r="C89" s="6" t="s">
@@ -6789,10 +6819,10 @@
         <v>14</v>
       </c>
       <c r="I89" s="7" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="J89" s="22" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="K89" s="6" t="b">
         <v>0</v>
@@ -6803,11 +6833,11 @@
     </row>
     <row r="90" spans="1:12" ht="319" x14ac:dyDescent="0.35">
       <c r="A90" s="6" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="B90" s="6"/>
       <c r="C90" s="6" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D90" s="6" t="s">
         <v>11</v>
@@ -6823,10 +6853,10 @@
         <v>12</v>
       </c>
       <c r="I90" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J90" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K90" s="6" t="b">
         <v>0</v>
@@ -6837,11 +6867,11 @@
     </row>
     <row r="91" spans="1:12" ht="319" x14ac:dyDescent="0.35">
       <c r="A91" s="23" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B91" s="23"/>
       <c r="C91" s="23" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D91" s="23" t="s">
         <v>11</v>
@@ -6854,13 +6884,13 @@
         <v>45000</v>
       </c>
       <c r="H91" s="23" t="s">
-        <v>277</v>
+        <v>358</v>
       </c>
       <c r="I91" s="7" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="J91" s="22" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="K91" s="6" t="b">
         <v>0</v>
@@ -6871,7 +6901,7 @@
     </row>
     <row r="92" spans="1:12" ht="391.5" x14ac:dyDescent="0.35">
       <c r="A92" s="23" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="B92" s="23"/>
       <c r="C92" s="23" t="s">
@@ -6891,10 +6921,10 @@
         <v>14</v>
       </c>
       <c r="I92" s="24" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="J92" s="22" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="K92" s="6" t="b">
         <v>0</v>
@@ -6905,11 +6935,11 @@
     </row>
     <row r="93" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A93" s="23" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B93" s="23"/>
       <c r="C93" s="23" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D93" s="23" t="s">
         <v>20</v>
@@ -6925,10 +6955,10 @@
         <v>14</v>
       </c>
       <c r="I93" s="7" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="J93" s="11" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="K93" s="6" t="b">
         <v>0</v>
@@ -6939,11 +6969,11 @@
     </row>
     <row r="94" spans="1:12" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A94" s="25" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="B94" s="25"/>
       <c r="C94" s="25" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D94" s="25" t="s">
         <v>20</v>
@@ -6959,10 +6989,10 @@
         <v>14</v>
       </c>
       <c r="I94" s="25" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="J94" s="26" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="K94" s="25" t="b">
         <v>0</v>
@@ -6973,11 +7003,11 @@
     </row>
     <row r="95" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A95" s="25" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B95" s="25"/>
       <c r="C95" s="25" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D95" s="25" t="s">
         <v>20</v>
@@ -6990,13 +7020,13 @@
         <v>15000</v>
       </c>
       <c r="H95" s="25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I95" s="26" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="J95" s="27" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="K95" s="25" t="b">
         <v>0</v>
@@ -7007,11 +7037,11 @@
     </row>
     <row r="96" spans="1:12" ht="261" x14ac:dyDescent="0.35">
       <c r="A96" s="25" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="B96" s="25"/>
       <c r="C96" s="25" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D96" s="25" t="s">
         <v>20</v>
@@ -7027,10 +7057,10 @@
         <v>14</v>
       </c>
       <c r="I96" s="25" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="J96" s="27" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="K96" s="25" t="b">
         <v>0</v>
@@ -7041,30 +7071,30 @@
     </row>
     <row r="97" spans="1:12" ht="174" x14ac:dyDescent="0.35">
       <c r="A97" s="25" t="s">
-        <v>306</v>
+        <v>370</v>
       </c>
       <c r="B97" s="25"/>
       <c r="C97" s="25" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D97" s="25" t="s">
         <v>20</v>
       </c>
       <c r="E97" s="25">
-        <v>24000</v>
+        <v>25000</v>
       </c>
       <c r="F97" s="25"/>
       <c r="G97" s="25">
-        <v>36000</v>
+        <v>37500</v>
       </c>
       <c r="H97" s="25" t="s">
         <v>14</v>
       </c>
       <c r="I97" s="25" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="J97" s="26" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="K97" s="25" t="b">
         <v>0</v>
@@ -7075,11 +7105,11 @@
     </row>
     <row r="98" spans="1:12" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A98" s="25" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B98" s="25"/>
       <c r="C98" s="25" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D98" s="25" t="s">
         <v>20</v>
@@ -7095,10 +7125,10 @@
         <v>14</v>
       </c>
       <c r="I98" s="26" t="s">
+        <v>304</v>
+      </c>
+      <c r="J98" s="26" t="s">
         <v>310</v>
-      </c>
-      <c r="J98" s="26" t="s">
-        <v>316</v>
       </c>
       <c r="K98" s="25" t="b">
         <v>0</v>
@@ -7109,11 +7139,11 @@
     </row>
     <row r="99" spans="1:12" ht="319" x14ac:dyDescent="0.35">
       <c r="A99" s="25" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="B99" s="25"/>
       <c r="C99" s="25" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D99" s="25" t="s">
         <v>20</v>
@@ -7129,10 +7159,10 @@
         <v>14</v>
       </c>
       <c r="I99" s="26" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="J99" s="26" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="K99" s="25" t="b">
         <v>0</v>
@@ -7143,11 +7173,11 @@
     </row>
     <row r="100" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A100" s="25" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="B100" s="25"/>
       <c r="C100" s="25" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D100" s="25" t="s">
         <v>20</v>
@@ -7163,10 +7193,10 @@
         <v>14</v>
       </c>
       <c r="I100" s="26" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="J100" s="26" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="K100" s="25" t="b">
         <v>0</v>
@@ -7177,11 +7207,11 @@
     </row>
     <row r="101" spans="1:12" ht="391.5" x14ac:dyDescent="0.35">
       <c r="A101" s="28" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="B101" s="28"/>
       <c r="C101" s="28" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D101" s="28" t="s">
         <v>20</v>
@@ -7197,10 +7227,10 @@
         <v>14</v>
       </c>
       <c r="I101" s="29" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="J101" s="29" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="K101" s="28" t="b">
         <v>0</v>
@@ -7211,11 +7241,11 @@
     </row>
     <row r="102" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A102" s="25" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="B102" s="25"/>
       <c r="C102" s="25" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D102" s="25" t="s">
         <v>20</v>
@@ -7231,10 +7261,10 @@
         <v>14</v>
       </c>
       <c r="I102" s="26" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="J102" s="26" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="K102" s="25" t="b">
         <v>0</v>
@@ -7245,11 +7275,11 @@
     </row>
     <row r="103" spans="1:12" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A103" s="28" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="B103" s="28"/>
       <c r="C103" s="28" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D103" s="28" t="s">
         <v>11</v>
@@ -7265,10 +7295,10 @@
         <v>14</v>
       </c>
       <c r="I103" s="28" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="J103" s="29" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="K103" s="28" t="b">
         <v>0</v>
@@ -7279,11 +7309,11 @@
     </row>
     <row r="104" spans="1:12" ht="391.5" x14ac:dyDescent="0.35">
       <c r="A104" s="28" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="B104" s="28"/>
       <c r="C104" s="28" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D104" s="28" t="s">
         <v>11</v>
@@ -7299,10 +7329,10 @@
         <v>14</v>
       </c>
       <c r="I104" s="29" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="J104" s="29" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="K104" s="28" t="b">
         <v>0</v>
@@ -7313,11 +7343,11 @@
     </row>
     <row r="105" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A105" s="25" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="B105" s="25"/>
       <c r="C105" s="25" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D105" s="25" t="s">
         <v>20</v>
@@ -7333,10 +7363,10 @@
         <v>14</v>
       </c>
       <c r="I105" s="26" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="J105" s="26" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="K105" s="25" t="b">
         <v>0</v>
@@ -7347,11 +7377,11 @@
     </row>
     <row r="106" spans="1:12" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A106" s="25" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="B106" s="25"/>
       <c r="C106" s="25" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D106" s="25" t="s">
         <v>20</v>
@@ -7367,10 +7397,10 @@
         <v>14</v>
       </c>
       <c r="I106" s="25" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="J106" s="26" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="K106" s="25" t="b">
         <v>0</v>
@@ -7381,11 +7411,11 @@
     </row>
     <row r="107" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A107" s="28" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="B107" s="28"/>
       <c r="C107" s="28" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D107" s="28" t="s">
         <v>11</v>
@@ -7401,10 +7431,10 @@
         <v>14</v>
       </c>
       <c r="I107" s="29" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="J107" s="29" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="K107" s="28" t="b">
         <v>0</v>
@@ -7415,11 +7445,11 @@
     </row>
     <row r="108" spans="1:12" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A108" s="28" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="B108" s="28"/>
       <c r="C108" s="28" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D108" s="28" t="s">
         <v>11</v>
@@ -7435,10 +7465,10 @@
         <v>14</v>
       </c>
       <c r="I108" s="28" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="J108" s="29" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="K108" s="28" t="b">
         <v>0</v>
@@ -7449,11 +7479,11 @@
     </row>
     <row r="109" spans="1:12" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A109" s="28" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="B109" s="28"/>
       <c r="C109" s="28" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D109" s="28" t="s">
         <v>11</v>
@@ -7469,10 +7499,10 @@
         <v>14</v>
       </c>
       <c r="I109" s="29" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="J109" s="29" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="K109" s="28" t="b">
         <v>0</v>
@@ -7483,11 +7513,11 @@
     </row>
     <row r="110" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A110" s="25" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="B110" s="25"/>
       <c r="C110" s="25" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D110" s="25" t="s">
         <v>26</v>
@@ -7503,10 +7533,10 @@
         <v>14</v>
       </c>
       <c r="I110" s="26" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="J110" s="26" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="K110" s="25" t="b">
         <v>0</v>
@@ -7517,11 +7547,11 @@
     </row>
     <row r="111" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A111" s="25" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="B111" s="25"/>
       <c r="C111" s="25" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D111" s="25" t="s">
         <v>26</v>
@@ -7537,10 +7567,10 @@
         <v>14</v>
       </c>
       <c r="I111" s="26" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="J111" s="26" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="K111" s="25" t="b">
         <v>0</v>
@@ -7551,11 +7581,11 @@
     </row>
     <row r="112" spans="1:12" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A112" s="25" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="B112" s="25"/>
       <c r="C112" s="25" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D112" s="25" t="s">
         <v>20</v>
@@ -7571,10 +7601,10 @@
         <v>14</v>
       </c>
       <c r="I112" s="26" t="s">
+        <v>304</v>
+      </c>
+      <c r="J112" s="26" t="s">
         <v>310</v>
-      </c>
-      <c r="J112" s="26" t="s">
-        <v>316</v>
       </c>
       <c r="K112" s="25" t="b">
         <v>0</v>
@@ -7585,11 +7615,11 @@
     </row>
     <row r="113" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A113" s="25" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="B113" s="25"/>
       <c r="C113" s="25" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D113" s="25" t="s">
         <v>11</v>
@@ -7605,10 +7635,10 @@
         <v>14</v>
       </c>
       <c r="I113" s="26" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="J113" s="26" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="K113" s="25" t="b">
         <v>0</v>
@@ -7619,11 +7649,11 @@
     </row>
     <row r="114" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A114" s="25" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="B114" s="25"/>
       <c r="C114" s="25" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D114" s="25" t="s">
         <v>26</v>
@@ -7639,10 +7669,10 @@
         <v>14</v>
       </c>
       <c r="I114" s="26" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="J114" s="26" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="K114" s="25" t="b">
         <v>0</v>
@@ -7653,11 +7683,11 @@
     </row>
     <row r="115" spans="1:12" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A115" s="25" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="B115" s="25"/>
       <c r="C115" s="25" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D115" s="25" t="s">
         <v>11</v>
@@ -7673,10 +7703,10 @@
         <v>14</v>
       </c>
       <c r="I115" s="26" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="J115" s="26" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="K115" s="25" t="b">
         <v>0</v>
@@ -7687,11 +7717,11 @@
     </row>
     <row r="116" spans="1:12" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A116" s="25" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="B116" s="25"/>
       <c r="C116" s="25" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D116" s="25" t="s">
         <v>11</v>
@@ -7704,18 +7734,52 @@
         <v>34000</v>
       </c>
       <c r="H116" s="25" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="I116" s="26" t="s">
+        <v>359</v>
+      </c>
+      <c r="J116" s="26" t="s">
+        <v>360</v>
+      </c>
+      <c r="K116" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="L116" s="25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" ht="290" x14ac:dyDescent="0.35">
+      <c r="A117" s="30" t="s">
         <v>366</v>
       </c>
-      <c r="J116" s="26" t="s">
+      <c r="B117" s="30"/>
+      <c r="C117" s="30" t="s">
+        <v>173</v>
+      </c>
+      <c r="D117" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="E117" s="30">
+        <v>26000</v>
+      </c>
+      <c r="F117" s="30"/>
+      <c r="G117" s="30">
+        <v>37500</v>
+      </c>
+      <c r="H117" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="I117" s="31" t="s">
         <v>367</v>
       </c>
-      <c r="K116" s="25" t="b">
-        <v>0</v>
-      </c>
-      <c r="L116" s="25" t="b">
+      <c r="J117" s="31" t="s">
+        <v>368</v>
+      </c>
+      <c r="K117" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="L117" s="30" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>